<commit_message>
Excel historico de operaciones
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoanalistas-my.sharepoint.com/personal/jpuerta_afi_es/Documents/Documentos/Master Quant/Gestión de activos/Trabajo gestión cuantitativa/Trabajo_gestion_cuantitativa/Envíos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1072D50-69C3-454B-AE54-75C8AB0F6E00}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{446651A5-453F-4530-B739-1DF7A9610F2B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="4575" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
+    <sheet name="Valor cartera" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -108,6 +109,9 @@
   </si>
   <si>
     <t>COMPRA</t>
+  </si>
+  <si>
+    <t>Valor cartera</t>
   </si>
 </sst>
 </file>
@@ -170,7 +174,44 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Amasis MT Pro"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -181,6 +222,22 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G17" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:G17" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
+    <tableColumn id="3" xr3:uid="{A21132F4-DD79-4C51-BEA4-4132F3EE35CB}" name="Acción"/>
+    <tableColumn id="4" xr3:uid="{6F333961-151C-4394-89A0-8580A62F023E}" name="Cantidad"/>
+    <tableColumn id="5" xr3:uid="{42F80897-162E-4CCE-9055-2FE010A8018C}" name="Precio" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -411,7 +468,7 @@
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="16.125" customWidth="1"/>
-    <col min="7" max="7" width="17.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.75" customWidth="1"/>
     <col min="9" max="9" width="11.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -847,6 +904,39 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="G19" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A40DD99D-6D96-4747-86B3-66E6AFFFF3C9}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>46093</v>
+      </c>
+      <c r="B2">
+        <v>10000000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Actualización tras las órdenes del 20 de marzo
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoanalistas-my.sharepoint.com/personal/jpuerta_afi_es/Documents/Documentos/Master Quant/Gestión de activos/Trabajo gestión cuantitativa/Trabajo_gestion_cuantitativa/Envíos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{446651A5-453F-4530-B739-1DF7A9610F2B}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A952E4C5-BADB-4AE3-9EEA-E4583FE29876}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="4575" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
@@ -36,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -112,14 +134,30 @@
   </si>
   <si>
     <t>Valor cartera</t>
+  </si>
+  <si>
+    <t>ENI.MI</t>
+  </si>
+  <si>
+    <t>VENTA</t>
+  </si>
+  <si>
+    <t>RMS.PA</t>
+  </si>
+  <si>
+    <t>SGO.PA</t>
+  </si>
+  <si>
+    <t>CASH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -164,17 +202,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -199,18 +250,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -224,17 +263,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G17" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:G17" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G36" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:G36" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
     <tableColumn id="3" xr3:uid="{A21132F4-DD79-4C51-BEA4-4132F3EE35CB}" name="Acción"/>
     <tableColumn id="4" xr3:uid="{6F333961-151C-4394-89A0-8580A62F023E}" name="Cantidad"/>
-    <tableColumn id="5" xr3:uid="{42F80897-162E-4CCE-9055-2FE010A8018C}" name="Precio" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{42F80897-162E-4CCE-9055-2FE010A8018C}" name="Precio" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -463,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -497,25 +540,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
-        <v>46093</v>
+        <v>46092</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>23</v>
       </c>
       <c r="D2">
-        <v>564</v>
+        <v>10000000</v>
       </c>
       <c r="E2" s="2">
-        <v>1180.40002441406</v>
+        <v>1</v>
       </c>
       <c r="F2" s="2">
-        <v>1.1803999999999999</v>
+        <v>0</v>
       </c>
       <c r="G2" s="2">
-        <v>1181.5804000000001</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -525,22 +568,22 @@
         <v>46093</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
       </c>
       <c r="D3">
-        <v>4362</v>
+        <v>564</v>
       </c>
       <c r="E3" s="2">
-        <v>152.64999389648401</v>
+        <v>1180.40002441406</v>
       </c>
       <c r="F3" s="2">
-        <v>0.15260000000000001</v>
+        <v>1.1803999999999999</v>
       </c>
       <c r="G3" s="2">
-        <v>152.80260000000001</v>
+        <v>1181.5804000000001</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
@@ -550,22 +593,22 @@
         <v>46093</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
       <c r="D4">
-        <v>36623</v>
+        <v>4362</v>
       </c>
       <c r="E4" s="2">
-        <v>18.184999465942301</v>
+        <v>152.64999389648401</v>
       </c>
       <c r="F4" s="2">
-        <v>1.8200000000000001E-2</v>
+        <v>0.15260000000000001</v>
       </c>
       <c r="G4" s="2">
-        <v>18.203199999999999</v>
+        <v>152.80260000000001</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -575,22 +618,22 @@
         <v>46093</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
       </c>
       <c r="D5">
-        <v>4716</v>
+        <v>36623</v>
       </c>
       <c r="E5" s="2">
-        <v>141.19999694824199</v>
+        <v>18.184999465942301</v>
       </c>
       <c r="F5" s="2">
-        <v>0.14119999999999999</v>
+        <v>1.8200000000000001E-2</v>
       </c>
       <c r="G5" s="2">
-        <v>141.34119999999999</v>
+        <v>18.203199999999999</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -600,22 +643,22 @@
         <v>46093</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
       </c>
       <c r="D6">
-        <v>14659</v>
+        <v>4716</v>
       </c>
       <c r="E6" s="2">
-        <v>45.430000305175703</v>
+        <v>141.19999694824199</v>
       </c>
       <c r="F6" s="2">
-        <v>4.5400000000000003E-2</v>
+        <v>0.14119999999999999</v>
       </c>
       <c r="G6" s="2">
-        <v>45.4754</v>
+        <v>141.34119999999999</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -625,22 +668,22 @@
         <v>46093</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
       </c>
       <c r="D7">
-        <v>3987</v>
+        <v>14659</v>
       </c>
       <c r="E7" s="2">
-        <v>167.02000427246</v>
+        <v>45.430000305175703</v>
       </c>
       <c r="F7" s="2">
-        <v>0.16700000000000001</v>
+        <v>4.5400000000000003E-2</v>
       </c>
       <c r="G7" s="2">
-        <v>167.18700000000001</v>
+        <v>45.4754</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -650,22 +693,22 @@
         <v>46093</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
         <v>23</v>
       </c>
       <c r="D8">
-        <v>3159</v>
+        <v>3987</v>
       </c>
       <c r="E8" s="2">
-        <v>210.80000305175699</v>
+        <v>167.02000427246</v>
       </c>
       <c r="F8" s="2">
-        <v>0.21079999999999999</v>
+        <v>0.16700000000000001</v>
       </c>
       <c r="G8" s="2">
-        <v>211.01079999999999</v>
+        <v>167.18700000000001</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -675,22 +718,22 @@
         <v>46093</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
         <v>23</v>
       </c>
       <c r="D9">
-        <v>2276</v>
+        <v>3159</v>
       </c>
       <c r="E9" s="2">
-        <v>292.600006103515</v>
+        <v>210.80000305175699</v>
       </c>
       <c r="F9" s="2">
-        <v>0.29260000000000003</v>
+        <v>0.21079999999999999</v>
       </c>
       <c r="G9" s="2">
-        <v>292.89260000000002</v>
+        <v>211.01079999999999</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -700,22 +743,22 @@
         <v>46093</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
       </c>
       <c r="D10">
-        <v>9919</v>
+        <v>2276</v>
       </c>
       <c r="E10" s="2">
-        <v>67.139999389648395</v>
+        <v>292.600006103515</v>
       </c>
       <c r="F10" s="2">
-        <v>6.7100000000000007E-2</v>
+        <v>0.29260000000000003</v>
       </c>
       <c r="G10" s="2">
-        <v>67.207099999999997</v>
+        <v>292.89260000000002</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -725,22 +768,22 @@
         <v>46093</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
         <v>23</v>
       </c>
       <c r="D11">
-        <v>17020</v>
+        <v>9919</v>
       </c>
       <c r="E11" s="2">
-        <v>39.130001068115199</v>
+        <v>67.139999389648395</v>
       </c>
       <c r="F11" s="2">
-        <v>3.9100000000000003E-2</v>
+        <v>6.7100000000000007E-2</v>
       </c>
       <c r="G11" s="2">
-        <v>39.1691</v>
+        <v>67.207099999999997</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -750,22 +793,22 @@
         <v>46093</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
         <v>23</v>
       </c>
       <c r="D12">
-        <v>726</v>
+        <v>17020</v>
       </c>
       <c r="E12" s="2">
-        <v>917.29998779296795</v>
+        <v>39.130001068115199</v>
       </c>
       <c r="F12" s="2">
-        <v>0.9173</v>
+        <v>3.9100000000000003E-2</v>
       </c>
       <c r="G12" s="2">
-        <v>918.21730000000002</v>
+        <v>39.1691</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -775,22 +818,22 @@
         <v>46093</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" t="s">
         <v>23</v>
       </c>
       <c r="D13">
-        <v>25909</v>
+        <v>726</v>
       </c>
       <c r="E13" s="2">
-        <v>25.704999923706001</v>
+        <v>917.29998779296795</v>
       </c>
       <c r="F13" s="2">
-        <v>2.5700000000000001E-2</v>
+        <v>0.9173</v>
       </c>
       <c r="G13" s="2">
-        <v>25.730699999999999</v>
+        <v>918.21730000000002</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -800,22 +843,22 @@
         <v>46093</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
         <v>23</v>
       </c>
       <c r="D14">
-        <v>429</v>
+        <v>25909</v>
       </c>
       <c r="E14" s="2">
-        <v>1550.5</v>
+        <v>25.704999923706001</v>
       </c>
       <c r="F14" s="2">
-        <v>1.5505</v>
+        <v>2.5700000000000001E-2</v>
       </c>
       <c r="G14" s="2">
-        <v>1552.0505000000001</v>
+        <v>25.730699999999999</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -825,22 +868,22 @@
         <v>46093</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C15" t="s">
         <v>23</v>
       </c>
       <c r="D15">
-        <v>1081</v>
+        <v>429</v>
       </c>
       <c r="E15" s="2">
-        <v>616</v>
+        <v>1550.5</v>
       </c>
       <c r="F15" s="2">
-        <v>0.61599999999999999</v>
+        <v>1.5505</v>
       </c>
       <c r="G15" s="2">
-        <v>616.61599999999999</v>
+        <v>1552.0505000000001</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -850,22 +893,22 @@
         <v>46093</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
         <v>23</v>
       </c>
       <c r="D16">
-        <v>3871</v>
+        <v>1081</v>
       </c>
       <c r="E16" s="2">
-        <v>172.03999328613199</v>
+        <v>616</v>
       </c>
       <c r="F16" s="2">
-        <v>0.17199999999999999</v>
+        <v>0.61599999999999999</v>
       </c>
       <c r="G16" s="2">
-        <v>172.21199999999999</v>
+        <v>616.61599999999999</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -875,35 +918,465 @@
         <v>46093</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="3">
-        <v>366.96075312617717</v>
+      <c r="D17">
+        <v>3871</v>
       </c>
       <c r="E17" s="2">
-        <v>5.0297000000000001</v>
+        <v>172.03999328613199</v>
       </c>
       <c r="F17" s="2">
-        <v>0</v>
+        <v>0.17199999999999999</v>
       </c>
       <c r="G17" s="2">
-        <v>5.0297000000000001</v>
+        <v>172.21199999999999</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="A18" s="4">
+        <v>46093</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="3">
+        <v>366.96075312617717</v>
+      </c>
+      <c r="E18" s="2">
+        <v>5.0297000000000001</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>5.0297000000000001</v>
+      </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G19" s="2"/>
+      <c r="A19" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19">
+        <v>74</v>
+      </c>
+      <c r="E19" s="2">
+        <v>194.75</v>
+      </c>
+      <c r="F19" s="2">
+        <v>9.7375000000000003E-2</v>
+      </c>
+      <c r="G19" s="2">
+        <v>194.847375</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" s="2">
+        <v>863.5</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0.43175000000000002</v>
+      </c>
+      <c r="G20" s="2">
+        <v>863.93174999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21">
+        <v>1077</v>
+      </c>
+      <c r="E21" s="2">
+        <v>40.020000457763601</v>
+      </c>
+      <c r="F21" s="2">
+        <v>2.0010000228881799E-2</v>
+      </c>
+      <c r="G21" s="2">
+        <v>40.040010457992501</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22">
+        <v>112</v>
+      </c>
+      <c r="E22" s="2">
+        <v>140.75</v>
+      </c>
+      <c r="F22" s="2">
+        <v>7.0374999999999993E-2</v>
+      </c>
+      <c r="G22" s="2">
+        <v>140.82037499999899</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2">
+        <v>133.5</v>
+      </c>
+      <c r="F23" s="2">
+        <v>6.6750000000000004E-2</v>
+      </c>
+      <c r="G23" s="2">
+        <v>133.56674999999899</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24">
+        <v>24</v>
+      </c>
+      <c r="E24" s="2">
+        <v>273.79998779296801</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0.136899993896484</v>
+      </c>
+      <c r="G24" s="2">
+        <v>273.93688778686499</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25">
+        <v>107</v>
+      </c>
+      <c r="E25" s="2">
+        <v>153.82000732421801</v>
+      </c>
+      <c r="F25" s="2">
+        <v>7.6910003662109303E-2</v>
+      </c>
+      <c r="G25" s="2">
+        <v>153.89691732788</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26">
+        <v>380</v>
+      </c>
+      <c r="E26" s="2">
+        <v>1656</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.82799999999999996</v>
+      </c>
+      <c r="G26" s="2">
+        <v>1656.828</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27">
+        <v>26650</v>
+      </c>
+      <c r="E27" s="2">
+        <v>23.620000839233398</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1.18100004196167E-2</v>
+      </c>
+      <c r="G27" s="2">
+        <v>23.631810839652999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28">
+        <v>9246</v>
+      </c>
+      <c r="E28" s="2">
+        <v>68.080001831054602</v>
+      </c>
+      <c r="F28" s="2">
+        <v>3.4040000915527301E-2</v>
+      </c>
+      <c r="G28" s="2">
+        <v>68.114041831970198</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29">
+        <v>-294</v>
+      </c>
+      <c r="E29" s="2">
+        <v>65.440002441406193</v>
+      </c>
+      <c r="F29" s="2">
+        <v>3.27200012207031E-2</v>
+      </c>
+      <c r="G29" s="2">
+        <v>65.407282440185497</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30">
+        <v>-4</v>
+      </c>
+      <c r="E30" s="2">
+        <v>584.79998779296795</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0.29239999389648402</v>
+      </c>
+      <c r="G30" s="2">
+        <v>584.50758779907198</v>
+      </c>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31">
+        <v>-612</v>
+      </c>
+      <c r="E31" s="2">
+        <v>38.384998321533203</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1.91924991607666E-2</v>
+      </c>
+      <c r="G31" s="2">
+        <v>38.365805822372401</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32">
+        <v>-472</v>
+      </c>
+      <c r="E32" s="2">
+        <v>24.7600002288818</v>
+      </c>
+      <c r="F32" s="2">
+        <v>1.23800001144409E-2</v>
+      </c>
+      <c r="G32" s="2">
+        <v>24.7476202287673</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B33" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33">
+        <v>-36623</v>
+      </c>
+      <c r="E33" s="2">
+        <v>17.924999237060501</v>
+      </c>
+      <c r="F33" s="2">
+        <v>8.9624996185302692E-3</v>
+      </c>
+      <c r="G33" s="2">
+        <v>17.916036737441999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" t="s">
+        <v>26</v>
+      </c>
+      <c r="D34">
+        <v>-429</v>
+      </c>
+      <c r="E34" s="2">
+        <v>1503</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0.75149999999999995</v>
+      </c>
+      <c r="G34" s="2">
+        <v>1502.2484999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35">
+        <v>-5</v>
+      </c>
+      <c r="E35" s="2">
+        <v>1128.19995117187</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0.56409997558593705</v>
+      </c>
+      <c r="G35" s="2">
+        <v>1127.6358511962801</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B36" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" t="s">
+        <v>26</v>
+      </c>
+      <c r="D36">
+        <v>-3871</v>
+      </c>
+      <c r="E36" s="2">
+        <v>160.919998168945</v>
+      </c>
+      <c r="F36" s="2">
+        <v>8.04599990844726E-2</v>
+      </c>
+      <c r="G36" s="2">
+        <v>160.83953816985999</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -915,15 +1388,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A40DD99D-6D96-4747-86B3-66E6AFFFF3C9}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B1" t="s">
@@ -931,11 +1404,31 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>46093</v>
-      </c>
-      <c r="B2">
+      <c r="A2" s="4" cm="1">
+        <f t="array" ref="A2:A4">_xlfn.UNIQUE(Operaciones_table[Fecha])</f>
+        <v>46092</v>
+      </c>
+      <c r="B2" s="5" cm="1">
+        <f t="array" ref="B2">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A2),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A2))</f>
         <v>10000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>46093</v>
+      </c>
+      <c r="B3" s="5" cm="1">
+        <f t="array" ref="B3">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]=A3),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]=A3))</f>
+        <v>9990013.1860319264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B4" s="5" cm="1">
+        <f t="array" ref="B4">B3+SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A4),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A4))</f>
+        <v>9990691.4268346932</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ordenes 27 de marzo
perdon, se me olvido subirlo antes
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoanalistas-my.sharepoint.com/personal/jpuerta_afi_es/Documents/Documentos/Master Quant/Gestión de activos/Trabajo gestión cuantitativa/Trabajo_gestion_cuantitativa/Envíos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A952E4C5-BADB-4AE3-9EEA-E4583FE29876}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8367EFF3-4BA8-4C0A-AE75-DAE2BEAB5854}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -149,6 +149,30 @@
   </si>
   <si>
     <t>CASH</t>
+  </si>
+  <si>
+    <t>Precio actual</t>
+  </si>
+  <si>
+    <t>Ticker</t>
+  </si>
+  <si>
+    <t>IFX.DE</t>
+  </si>
+  <si>
+    <t>TTE.PA</t>
+  </si>
+  <si>
+    <t>UCG.MI</t>
+  </si>
+  <si>
+    <t>SAF.PA</t>
+  </si>
+  <si>
+    <t>INGA.AS</t>
+  </si>
+  <si>
+    <t>SAN.MC</t>
   </si>
 </sst>
 </file>
@@ -268,8 +292,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G36" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:G36" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G58" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:G58" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
@@ -506,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -1378,6 +1402,512 @@
         <v>160.83953816985999</v>
       </c>
     </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D37">
+        <v>5846</v>
+      </c>
+      <c r="E37" s="2">
+        <v>37.430000305175703</v>
+      </c>
+      <c r="F37" s="2">
+        <v>1.8715000152587799E-2</v>
+      </c>
+      <c r="G37" s="2">
+        <v>37.4487153053283</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38">
+        <v>34714</v>
+      </c>
+      <c r="E38" s="2">
+        <v>23.924999237060501</v>
+      </c>
+      <c r="F38" s="2">
+        <v>1.1962499618530201E-2</v>
+      </c>
+      <c r="G38" s="2">
+        <v>23.936961736678999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39">
+        <v>279</v>
+      </c>
+      <c r="E39" s="2">
+        <v>1146.40002441406</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0.57320001220703098</v>
+      </c>
+      <c r="G39" s="2">
+        <v>1146.97322442626</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B40" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40">
+        <v>221</v>
+      </c>
+      <c r="E40" s="2">
+        <v>1379.5</v>
+      </c>
+      <c r="F40" s="2">
+        <v>0.68974999999999997</v>
+      </c>
+      <c r="G40" s="2">
+        <v>1380.18975</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" t="s">
+        <v>23</v>
+      </c>
+      <c r="D41">
+        <v>18700</v>
+      </c>
+      <c r="E41" s="2">
+        <v>78.489997863769503</v>
+      </c>
+      <c r="F41" s="2">
+        <v>3.9244998931884698E-2</v>
+      </c>
+      <c r="G41" s="2">
+        <v>78.529242862701395</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B42" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42">
+        <v>12173</v>
+      </c>
+      <c r="E42" s="2">
+        <v>60.220001220703097</v>
+      </c>
+      <c r="F42" s="2">
+        <v>3.01100006103515E-2</v>
+      </c>
+      <c r="G42" s="2">
+        <v>60.250111221313396</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B43" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43">
+        <v>1724</v>
+      </c>
+      <c r="E43" s="2">
+        <v>278.39999389648398</v>
+      </c>
+      <c r="F43" s="2">
+        <v>0.13919999694824201</v>
+      </c>
+      <c r="G43" s="2">
+        <v>278.53919389343201</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B44" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44">
+        <v>34709</v>
+      </c>
+      <c r="E44" s="2">
+        <v>21.7199993133544</v>
+      </c>
+      <c r="F44" s="2">
+        <v>1.0859999656677201E-2</v>
+      </c>
+      <c r="G44" s="2">
+        <v>21.730859313011099</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B45" t="s">
+        <v>37</v>
+      </c>
+      <c r="C45" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45">
+        <v>56041</v>
+      </c>
+      <c r="E45" s="2">
+        <v>9.4020004272460902</v>
+      </c>
+      <c r="F45" s="2">
+        <v>4.7010002136230397E-3</v>
+      </c>
+      <c r="G45" s="2">
+        <v>9.4067014274597103</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B46" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46">
+        <v>-1609</v>
+      </c>
+      <c r="E46" s="2">
+        <v>38.259998321533203</v>
+      </c>
+      <c r="F46" s="2">
+        <v>1.91299991607666E-2</v>
+      </c>
+      <c r="G46" s="2">
+        <v>38.2408683223724</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B47" t="s">
+        <v>28</v>
+      </c>
+      <c r="C47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47">
+        <v>-1553</v>
+      </c>
+      <c r="E47" s="2">
+        <v>69.120002746582003</v>
+      </c>
+      <c r="F47" s="2">
+        <v>3.4560001373291002E-2</v>
+      </c>
+      <c r="G47" s="2">
+        <v>69.085442745208695</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B48" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48">
+        <v>-13938</v>
+      </c>
+      <c r="E48" s="2">
+        <v>24.915000915527301</v>
+      </c>
+      <c r="F48" s="2">
+        <v>1.2457500457763599E-2</v>
+      </c>
+      <c r="G48" s="2">
+        <v>24.902543415069498</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49">
+        <v>-2845</v>
+      </c>
+      <c r="E49" s="2">
+        <v>132.05000305175699</v>
+      </c>
+      <c r="F49" s="2">
+        <v>6.6025001525878896E-2</v>
+      </c>
+      <c r="G49" s="2">
+        <v>131.983978050231</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B50" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50">
+        <v>-15736</v>
+      </c>
+      <c r="E50" s="2">
+        <v>38.720001220703097</v>
+      </c>
+      <c r="F50" s="2">
+        <v>1.9360000610351501E-2</v>
+      </c>
+      <c r="G50" s="2">
+        <v>38.700641220092699</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51">
+        <v>-3233</v>
+      </c>
+      <c r="E51" s="2">
+        <v>194.80000305175699</v>
+      </c>
+      <c r="F51" s="2">
+        <v>9.7400001525878896E-2</v>
+      </c>
+      <c r="G51" s="2">
+        <v>194.702603050231</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B52" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52">
+        <v>-1077</v>
+      </c>
+      <c r="E52" s="2">
+        <v>607.40002441406205</v>
+      </c>
+      <c r="F52" s="2">
+        <v>0.30370001220703102</v>
+      </c>
+      <c r="G52" s="2">
+        <v>607.09632440185499</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B53" t="s">
+        <v>27</v>
+      </c>
+      <c r="C53" t="s">
+        <v>26</v>
+      </c>
+      <c r="D53">
+        <v>-380</v>
+      </c>
+      <c r="E53" s="2">
+        <v>1621.5</v>
+      </c>
+      <c r="F53" s="2">
+        <v>0.81074999999999997</v>
+      </c>
+      <c r="G53" s="2">
+        <v>1620.6892499999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B54" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" t="s">
+        <v>26</v>
+      </c>
+      <c r="D54">
+        <v>-9625</v>
+      </c>
+      <c r="E54" s="2">
+        <v>62.319999694824197</v>
+      </c>
+      <c r="F54" s="2">
+        <v>3.11599998474121E-2</v>
+      </c>
+      <c r="G54" s="2">
+        <v>62.288839694976801</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B55" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" t="s">
+        <v>26</v>
+      </c>
+      <c r="D55">
+        <v>-2300</v>
+      </c>
+      <c r="E55" s="2">
+        <v>278.29998779296801</v>
+      </c>
+      <c r="F55" s="2">
+        <v>0.139149993896484</v>
+      </c>
+      <c r="G55" s="2">
+        <v>278.160837799072</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B56" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" t="s">
+        <v>26</v>
+      </c>
+      <c r="D56">
+        <v>-4094</v>
+      </c>
+      <c r="E56" s="2">
+        <v>142.55999755859301</v>
+      </c>
+      <c r="F56" s="2">
+        <v>7.1279998779296805E-2</v>
+      </c>
+      <c r="G56" s="2">
+        <v>142.48871755981401</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C57" t="s">
+        <v>26</v>
+      </c>
+      <c r="D57">
+        <v>-431</v>
+      </c>
+      <c r="E57" s="2">
+        <v>855.5</v>
+      </c>
+      <c r="F57" s="2">
+        <v>0.42775000000000002</v>
+      </c>
+      <c r="G57" s="2">
+        <v>855.07225000000005</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" t="s">
+        <v>26</v>
+      </c>
+      <c r="D58">
+        <v>-321</v>
+      </c>
+      <c r="E58" s="2">
+        <v>144.39999389648401</v>
+      </c>
+      <c r="F58" s="2">
+        <v>7.2199996948242195E-2</v>
+      </c>
+      <c r="G58" s="2">
+        <v>144.327793899536</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -1388,32 +1918,42 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A40DD99D-6D96-4747-86B3-66E6AFFFF3C9}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" cm="1">
-        <f t="array" ref="A2:A4">_xlfn.UNIQUE(Operaciones_table[Fecha])</f>
+        <f t="array" ref="A2:A5">_xlfn.UNIQUE(Operaciones_table[Fecha])</f>
         <v>46092</v>
       </c>
       <c r="B2" s="5" cm="1">
         <f t="array" ref="B2">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A2),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A2))</f>
         <v>10000000</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>46093</v>
       </c>
@@ -1422,13 +1962,18 @@
         <v>9990013.1860319264</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>46101</v>
       </c>
       <c r="B4" s="5" cm="1">
         <f t="array" ref="B4">B3+SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A4),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A4))</f>
         <v>9990691.4268346932</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>46108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
envío 3 de abril
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoanalistas-my.sharepoint.com/personal/jpuerta_afi_es/Documents/Documentos/Master Quant/Gestión de activos/Trabajo gestión cuantitativa/Trabajo_gestion_cuantitativa/Envíos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Master Quant\Gestión de activos\Trabajo gestión cuantitativa\Trabajo_gestion_cuantitativa\Trabajo_gestion_cuantitativa\Envíos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="8_{F17BE316-1B00-40D4-ADE9-8559E06525B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8367EFF3-4BA8-4C0A-AE75-DAE2BEAB5854}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B4E8EB-8366-4071-B11E-B048FB6ABFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
@@ -21,30 +21,19 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -59,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -226,20 +215,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
@@ -292,16 +282,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G58" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:G58" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G74" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:G74" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
     <tableColumn id="3" xr3:uid="{A21132F4-DD79-4C51-BEA4-4132F3EE35CB}" name="Acción"/>
     <tableColumn id="4" xr3:uid="{6F333961-151C-4394-89A0-8580A62F023E}" name="Cantidad"/>
     <tableColumn id="5" xr3:uid="{42F80897-162E-4CCE-9055-2FE010A8018C}" name="Precio" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -530,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -578,8 +568,8 @@
       <c r="E2" s="2">
         <v>1</v>
       </c>
-      <c r="F2" s="2">
-        <v>0</v>
+      <c r="F2" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G2" s="2">
         <v>1</v>
@@ -603,8 +593,8 @@
       <c r="E3" s="2">
         <v>1180.40002441406</v>
       </c>
-      <c r="F3" s="2">
-        <v>1.1803999999999999</v>
+      <c r="F3" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G3" s="2">
         <v>1181.5804000000001</v>
@@ -628,8 +618,8 @@
       <c r="E4" s="2">
         <v>152.64999389648401</v>
       </c>
-      <c r="F4" s="2">
-        <v>0.15260000000000001</v>
+      <c r="F4" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G4" s="2">
         <v>152.80260000000001</v>
@@ -653,8 +643,8 @@
       <c r="E5" s="2">
         <v>18.184999465942301</v>
       </c>
-      <c r="F5" s="2">
-        <v>1.8200000000000001E-2</v>
+      <c r="F5" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G5" s="2">
         <v>18.203199999999999</v>
@@ -678,8 +668,8 @@
       <c r="E6" s="2">
         <v>141.19999694824199</v>
       </c>
-      <c r="F6" s="2">
-        <v>0.14119999999999999</v>
+      <c r="F6" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G6" s="2">
         <v>141.34119999999999</v>
@@ -703,8 +693,8 @@
       <c r="E7" s="2">
         <v>45.430000305175703</v>
       </c>
-      <c r="F7" s="2">
-        <v>4.5400000000000003E-2</v>
+      <c r="F7" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G7" s="2">
         <v>45.4754</v>
@@ -728,8 +718,8 @@
       <c r="E8" s="2">
         <v>167.02000427246</v>
       </c>
-      <c r="F8" s="2">
-        <v>0.16700000000000001</v>
+      <c r="F8" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G8" s="2">
         <v>167.18700000000001</v>
@@ -753,8 +743,8 @@
       <c r="E9" s="2">
         <v>210.80000305175699</v>
       </c>
-      <c r="F9" s="2">
-        <v>0.21079999999999999</v>
+      <c r="F9" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G9" s="2">
         <v>211.01079999999999</v>
@@ -778,8 +768,8 @@
       <c r="E10" s="2">
         <v>292.600006103515</v>
       </c>
-      <c r="F10" s="2">
-        <v>0.29260000000000003</v>
+      <c r="F10" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G10" s="2">
         <v>292.89260000000002</v>
@@ -803,8 +793,8 @@
       <c r="E11" s="2">
         <v>67.139999389648395</v>
       </c>
-      <c r="F11" s="2">
-        <v>6.7100000000000007E-2</v>
+      <c r="F11" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G11" s="2">
         <v>67.207099999999997</v>
@@ -828,8 +818,8 @@
       <c r="E12" s="2">
         <v>39.130001068115199</v>
       </c>
-      <c r="F12" s="2">
-        <v>3.9100000000000003E-2</v>
+      <c r="F12" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G12" s="2">
         <v>39.1691</v>
@@ -853,8 +843,8 @@
       <c r="E13" s="2">
         <v>917.29998779296795</v>
       </c>
-      <c r="F13" s="2">
-        <v>0.9173</v>
+      <c r="F13" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G13" s="2">
         <v>918.21730000000002</v>
@@ -878,8 +868,8 @@
       <c r="E14" s="2">
         <v>25.704999923706001</v>
       </c>
-      <c r="F14" s="2">
-        <v>2.5700000000000001E-2</v>
+      <c r="F14" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G14" s="2">
         <v>25.730699999999999</v>
@@ -903,8 +893,8 @@
       <c r="E15" s="2">
         <v>1550.5</v>
       </c>
-      <c r="F15" s="2">
-        <v>1.5505</v>
+      <c r="F15" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G15" s="2">
         <v>1552.0505000000001</v>
@@ -928,8 +918,8 @@
       <c r="E16" s="2">
         <v>616</v>
       </c>
-      <c r="F16" s="2">
-        <v>0.61599999999999999</v>
+      <c r="F16" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G16" s="2">
         <v>616.61599999999999</v>
@@ -953,8 +943,8 @@
       <c r="E17" s="2">
         <v>172.03999328613199</v>
       </c>
-      <c r="F17" s="2">
-        <v>0.17199999999999999</v>
+      <c r="F17" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G17" s="2">
         <v>172.21199999999999</v>
@@ -978,8 +968,8 @@
       <c r="E18" s="2">
         <v>5.0297000000000001</v>
       </c>
-      <c r="F18" s="2">
-        <v>0</v>
+      <c r="F18" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G18" s="2">
         <v>5.0297000000000001</v>
@@ -1003,8 +993,8 @@
       <c r="E19" s="2">
         <v>194.75</v>
       </c>
-      <c r="F19" s="2">
-        <v>9.7375000000000003E-2</v>
+      <c r="F19" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G19" s="2">
         <v>194.847375</v>
@@ -1026,8 +1016,8 @@
       <c r="E20" s="2">
         <v>863.5</v>
       </c>
-      <c r="F20" s="2">
-        <v>0.43175000000000002</v>
+      <c r="F20" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G20" s="2">
         <v>863.93174999999997</v>
@@ -1049,8 +1039,8 @@
       <c r="E21" s="2">
         <v>40.020000457763601</v>
       </c>
-      <c r="F21" s="2">
-        <v>2.0010000228881799E-2</v>
+      <c r="F21" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G21" s="2">
         <v>40.040010457992501</v>
@@ -1072,8 +1062,8 @@
       <c r="E22" s="2">
         <v>140.75</v>
       </c>
-      <c r="F22" s="2">
-        <v>7.0374999999999993E-2</v>
+      <c r="F22" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G22" s="2">
         <v>140.82037499999899</v>
@@ -1095,8 +1085,8 @@
       <c r="E23" s="2">
         <v>133.5</v>
       </c>
-      <c r="F23" s="2">
-        <v>6.6750000000000004E-2</v>
+      <c r="F23" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G23" s="2">
         <v>133.56674999999899</v>
@@ -1118,8 +1108,8 @@
       <c r="E24" s="2">
         <v>273.79998779296801</v>
       </c>
-      <c r="F24" s="2">
-        <v>0.136899993896484</v>
+      <c r="F24" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G24" s="2">
         <v>273.93688778686499</v>
@@ -1141,8 +1131,8 @@
       <c r="E25" s="2">
         <v>153.82000732421801</v>
       </c>
-      <c r="F25" s="2">
-        <v>7.6910003662109303E-2</v>
+      <c r="F25" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G25" s="2">
         <v>153.89691732788</v>
@@ -1164,8 +1154,8 @@
       <c r="E26" s="2">
         <v>1656</v>
       </c>
-      <c r="F26" s="2">
-        <v>0.82799999999999996</v>
+      <c r="F26" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G26" s="2">
         <v>1656.828</v>
@@ -1187,8 +1177,8 @@
       <c r="E27" s="2">
         <v>23.620000839233398</v>
       </c>
-      <c r="F27" s="2">
-        <v>1.18100004196167E-2</v>
+      <c r="F27" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G27" s="2">
         <v>23.631810839652999</v>
@@ -1210,8 +1200,8 @@
       <c r="E28" s="2">
         <v>68.080001831054602</v>
       </c>
-      <c r="F28" s="2">
-        <v>3.4040000915527301E-2</v>
+      <c r="F28" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G28" s="2">
         <v>68.114041831970198</v>
@@ -1233,8 +1223,8 @@
       <c r="E29" s="2">
         <v>65.440002441406193</v>
       </c>
-      <c r="F29" s="2">
-        <v>3.27200012207031E-2</v>
+      <c r="F29" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G29" s="2">
         <v>65.407282440185497</v>
@@ -1256,8 +1246,8 @@
       <c r="E30" s="2">
         <v>584.79998779296795</v>
       </c>
-      <c r="F30" s="2">
-        <v>0.29239999389648402</v>
+      <c r="F30" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G30" s="2">
         <v>584.50758779907198</v>
@@ -1280,8 +1270,8 @@
       <c r="E31" s="2">
         <v>38.384998321533203</v>
       </c>
-      <c r="F31" s="2">
-        <v>1.91924991607666E-2</v>
+      <c r="F31" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G31" s="2">
         <v>38.365805822372401</v>
@@ -1303,8 +1293,8 @@
       <c r="E32" s="2">
         <v>24.7600002288818</v>
       </c>
-      <c r="F32" s="2">
-        <v>1.23800001144409E-2</v>
+      <c r="F32" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G32" s="2">
         <v>24.7476202287673</v>
@@ -1326,8 +1316,8 @@
       <c r="E33" s="2">
         <v>17.924999237060501</v>
       </c>
-      <c r="F33" s="2">
-        <v>8.9624996185302692E-3</v>
+      <c r="F33" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G33" s="2">
         <v>17.916036737441999</v>
@@ -1349,8 +1339,8 @@
       <c r="E34" s="2">
         <v>1503</v>
       </c>
-      <c r="F34" s="2">
-        <v>0.75149999999999995</v>
+      <c r="F34" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G34" s="2">
         <v>1502.2484999999999</v>
@@ -1372,8 +1362,8 @@
       <c r="E35" s="2">
         <v>1128.19995117187</v>
       </c>
-      <c r="F35" s="2">
-        <v>0.56409997558593705</v>
+      <c r="F35" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G35" s="2">
         <v>1127.6358511962801</v>
@@ -1395,8 +1385,8 @@
       <c r="E36" s="2">
         <v>160.919998168945</v>
       </c>
-      <c r="F36" s="2">
-        <v>8.04599990844726E-2</v>
+      <c r="F36" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G36" s="2">
         <v>160.83953816985999</v>
@@ -1418,8 +1408,8 @@
       <c r="E37" s="2">
         <v>37.430000305175703</v>
       </c>
-      <c r="F37" s="2">
-        <v>1.8715000152587799E-2</v>
+      <c r="F37" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G37" s="2">
         <v>37.4487153053283</v>
@@ -1441,8 +1431,8 @@
       <c r="E38" s="2">
         <v>23.924999237060501</v>
       </c>
-      <c r="F38" s="2">
-        <v>1.1962499618530201E-2</v>
+      <c r="F38" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G38" s="2">
         <v>23.936961736678999</v>
@@ -1464,8 +1454,8 @@
       <c r="E39" s="2">
         <v>1146.40002441406</v>
       </c>
-      <c r="F39" s="2">
-        <v>0.57320001220703098</v>
+      <c r="F39" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G39" s="2">
         <v>1146.97322442626</v>
@@ -1487,8 +1477,8 @@
       <c r="E40" s="2">
         <v>1379.5</v>
       </c>
-      <c r="F40" s="2">
-        <v>0.68974999999999997</v>
+      <c r="F40" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G40" s="2">
         <v>1380.18975</v>
@@ -1510,8 +1500,8 @@
       <c r="E41" s="2">
         <v>78.489997863769503</v>
       </c>
-      <c r="F41" s="2">
-        <v>3.9244998931884698E-2</v>
+      <c r="F41" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G41" s="2">
         <v>78.529242862701395</v>
@@ -1533,8 +1523,8 @@
       <c r="E42" s="2">
         <v>60.220001220703097</v>
       </c>
-      <c r="F42" s="2">
-        <v>3.01100006103515E-2</v>
+      <c r="F42" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G42" s="2">
         <v>60.250111221313396</v>
@@ -1556,8 +1546,8 @@
       <c r="E43" s="2">
         <v>278.39999389648398</v>
       </c>
-      <c r="F43" s="2">
-        <v>0.13919999694824201</v>
+      <c r="F43" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G43" s="2">
         <v>278.53919389343201</v>
@@ -1579,8 +1569,8 @@
       <c r="E44" s="2">
         <v>21.7199993133544</v>
       </c>
-      <c r="F44" s="2">
-        <v>1.0859999656677201E-2</v>
+      <c r="F44" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G44" s="2">
         <v>21.730859313011099</v>
@@ -1602,8 +1592,8 @@
       <c r="E45" s="2">
         <v>9.4020004272460902</v>
       </c>
-      <c r="F45" s="2">
-        <v>4.7010002136230397E-3</v>
+      <c r="F45" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G45" s="2">
         <v>9.4067014274597103</v>
@@ -1625,8 +1615,8 @@
       <c r="E46" s="2">
         <v>38.259998321533203</v>
       </c>
-      <c r="F46" s="2">
-        <v>1.91299991607666E-2</v>
+      <c r="F46" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G46" s="2">
         <v>38.2408683223724</v>
@@ -1648,8 +1638,8 @@
       <c r="E47" s="2">
         <v>69.120002746582003</v>
       </c>
-      <c r="F47" s="2">
-        <v>3.4560001373291002E-2</v>
+      <c r="F47" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G47" s="2">
         <v>69.085442745208695</v>
@@ -1671,8 +1661,8 @@
       <c r="E48" s="2">
         <v>24.915000915527301</v>
       </c>
-      <c r="F48" s="2">
-        <v>1.2457500457763599E-2</v>
+      <c r="F48" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G48" s="2">
         <v>24.902543415069498</v>
@@ -1694,8 +1684,8 @@
       <c r="E49" s="2">
         <v>132.05000305175699</v>
       </c>
-      <c r="F49" s="2">
-        <v>6.6025001525878896E-2</v>
+      <c r="F49" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G49" s="2">
         <v>131.983978050231</v>
@@ -1717,8 +1707,8 @@
       <c r="E50" s="2">
         <v>38.720001220703097</v>
       </c>
-      <c r="F50" s="2">
-        <v>1.9360000610351501E-2</v>
+      <c r="F50" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G50" s="2">
         <v>38.700641220092699</v>
@@ -1740,8 +1730,8 @@
       <c r="E51" s="2">
         <v>194.80000305175699</v>
       </c>
-      <c r="F51" s="2">
-        <v>9.7400001525878896E-2</v>
+      <c r="F51" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G51" s="2">
         <v>194.702603050231</v>
@@ -1763,8 +1753,8 @@
       <c r="E52" s="2">
         <v>607.40002441406205</v>
       </c>
-      <c r="F52" s="2">
-        <v>0.30370001220703102</v>
+      <c r="F52" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G52" s="2">
         <v>607.09632440185499</v>
@@ -1786,8 +1776,8 @@
       <c r="E53" s="2">
         <v>1621.5</v>
       </c>
-      <c r="F53" s="2">
-        <v>0.81074999999999997</v>
+      <c r="F53" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G53" s="2">
         <v>1620.6892499999999</v>
@@ -1809,8 +1799,8 @@
       <c r="E54" s="2">
         <v>62.319999694824197</v>
       </c>
-      <c r="F54" s="2">
-        <v>3.11599998474121E-2</v>
+      <c r="F54" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G54" s="2">
         <v>62.288839694976801</v>
@@ -1832,8 +1822,8 @@
       <c r="E55" s="2">
         <v>278.29998779296801</v>
       </c>
-      <c r="F55" s="2">
-        <v>0.139149993896484</v>
+      <c r="F55" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G55" s="2">
         <v>278.160837799072</v>
@@ -1855,8 +1845,8 @@
       <c r="E56" s="2">
         <v>142.55999755859301</v>
       </c>
-      <c r="F56" s="2">
-        <v>7.1279998779296805E-2</v>
+      <c r="F56" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G56" s="2">
         <v>142.48871755981401</v>
@@ -1878,8 +1868,8 @@
       <c r="E57" s="2">
         <v>855.5</v>
       </c>
-      <c r="F57" s="2">
-        <v>0.42775000000000002</v>
+      <c r="F57" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G57" s="2">
         <v>855.07225000000005</v>
@@ -1901,11 +1891,379 @@
       <c r="E58" s="2">
         <v>144.39999389648401</v>
       </c>
-      <c r="F58" s="2">
-        <v>7.2199996948242195E-2</v>
+      <c r="F58" s="6">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G58" s="2">
         <v>144.327793899536</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B59" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" t="s">
+        <v>23</v>
+      </c>
+      <c r="D59">
+        <v>7328</v>
+      </c>
+      <c r="E59" s="2">
+        <v>39.694999694824197</v>
+      </c>
+      <c r="F59" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G59" s="2">
+        <v>39.714847194671599</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B60" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" t="s">
+        <v>23</v>
+      </c>
+      <c r="D60">
+        <v>37957</v>
+      </c>
+      <c r="E60" s="2">
+        <v>18.770000457763601</v>
+      </c>
+      <c r="F60" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G60" s="2">
+        <v>18.7793854579925</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B61" t="s">
+        <v>12</v>
+      </c>
+      <c r="C61" t="s">
+        <v>23</v>
+      </c>
+      <c r="D61">
+        <v>782</v>
+      </c>
+      <c r="E61" s="2">
+        <v>295.5</v>
+      </c>
+      <c r="F61" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G61" s="2">
+        <v>295.64774999999997</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B62" t="s">
+        <v>35</v>
+      </c>
+      <c r="C62" t="s">
+        <v>23</v>
+      </c>
+      <c r="D62">
+        <v>246</v>
+      </c>
+      <c r="E62" s="2">
+        <v>287.29998779296801</v>
+      </c>
+      <c r="F62" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G62" s="2">
+        <v>287.443637786865</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B63" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" t="s">
+        <v>23</v>
+      </c>
+      <c r="D63">
+        <v>314</v>
+      </c>
+      <c r="E63" s="2">
+        <v>1161</v>
+      </c>
+      <c r="F63" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G63" s="2">
+        <v>1161.5805</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B64" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64" t="s">
+        <v>23</v>
+      </c>
+      <c r="D64">
+        <v>947</v>
+      </c>
+      <c r="E64" s="2">
+        <v>134.89999389648401</v>
+      </c>
+      <c r="F64" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G64" s="2">
+        <v>134.96744389343201</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B65" t="s">
+        <v>16</v>
+      </c>
+      <c r="C65" t="s">
+        <v>23</v>
+      </c>
+      <c r="D65">
+        <v>1216</v>
+      </c>
+      <c r="E65" s="2">
+        <v>25.674999237060501</v>
+      </c>
+      <c r="F65" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G65" s="2">
+        <v>25.687836736678999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B66" t="s">
+        <v>32</v>
+      </c>
+      <c r="C66" t="s">
+        <v>23</v>
+      </c>
+      <c r="D66">
+        <v>6143</v>
+      </c>
+      <c r="E66" s="2">
+        <v>38.959999084472599</v>
+      </c>
+      <c r="F66" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G66" s="2">
+        <v>38.979479084014798</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B67" t="s">
+        <v>33</v>
+      </c>
+      <c r="C67" t="s">
+        <v>23</v>
+      </c>
+      <c r="D67">
+        <v>2177</v>
+      </c>
+      <c r="E67" s="2">
+        <v>79.419998168945298</v>
+      </c>
+      <c r="F67" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G67" s="2">
+        <v>79.459708168029707</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B68" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68" t="s">
+        <v>26</v>
+      </c>
+      <c r="D68">
+        <v>-3861</v>
+      </c>
+      <c r="E68" s="2">
+        <v>70.519996643066406</v>
+      </c>
+      <c r="F68" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G68" s="2">
+        <v>70.4847366447448</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B69" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>26</v>
+      </c>
+      <c r="D69">
+        <v>-2461</v>
+      </c>
+      <c r="E69" s="2">
+        <v>149.69999694824199</v>
+      </c>
+      <c r="F69" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G69" s="2">
+        <v>149.62514694976801</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B70" t="s">
+        <v>34</v>
+      </c>
+      <c r="C70" t="s">
+        <v>26</v>
+      </c>
+      <c r="D70">
+        <v>-12173</v>
+      </c>
+      <c r="E70" s="2">
+        <v>62.659999847412102</v>
+      </c>
+      <c r="F70" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G70" s="2">
+        <v>62.628669847488403</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B71" t="s">
+        <v>36</v>
+      </c>
+      <c r="C71" t="s">
+        <v>26</v>
+      </c>
+      <c r="D71">
+        <v>-5905</v>
+      </c>
+      <c r="E71" s="2">
+        <v>22.944999694824201</v>
+      </c>
+      <c r="F71" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G71" s="2">
+        <v>22.933527194976801</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B72" t="s">
+        <v>25</v>
+      </c>
+      <c r="C72" t="s">
+        <v>26</v>
+      </c>
+      <c r="D72">
+        <v>-12852</v>
+      </c>
+      <c r="E72" s="2">
+        <v>24.684999465942301</v>
+      </c>
+      <c r="F72" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G72" s="2">
+        <v>24.672656966209399</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B73" t="s">
+        <v>17</v>
+      </c>
+      <c r="C73" t="s">
+        <v>26</v>
+      </c>
+      <c r="D73">
+        <v>-221</v>
+      </c>
+      <c r="E73" s="2">
+        <v>1570.5</v>
+      </c>
+      <c r="F73" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G73" s="2">
+        <v>1569.7147500000001</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="4">
+        <v>46115</v>
+      </c>
+      <c r="B74" t="s">
+        <v>37</v>
+      </c>
+      <c r="C74" t="s">
+        <v>26</v>
+      </c>
+      <c r="D74">
+        <v>-4227</v>
+      </c>
+      <c r="E74" s="2">
+        <v>9.8140001296996999</v>
+      </c>
+      <c r="F74" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G74" s="2">
+        <v>9.8090931296348494</v>
       </c>
     </row>
   </sheetData>
@@ -1938,13 +2296,13 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" cm="1">
-        <f t="array" ref="A2:A5">_xlfn.UNIQUE(Operaciones_table[Fecha])</f>
-        <v>46092</v>
-      </c>
-      <c r="B2" s="5" cm="1">
-        <f t="array" ref="B2">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A2),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A2))</f>
-        <v>10000000</v>
+      <c r="A2" s="4" t="e" cm="1">
+        <f t="array" aca="1" ref="A2:A5" ca="1">_xlfn.UNIQUE(Operaciones_table[Fecha])</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="B2" s="5" t="e" cm="1">
+        <f t="array" aca="1" ref="B2" ca="1">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A2),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A2))</f>
+        <v>#NAME?</v>
       </c>
       <c r="E2" t="s">
         <v>31</v>
@@ -1954,26 +2312,29 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>46093</v>
-      </c>
-      <c r="B3" s="5" cm="1">
-        <f t="array" ref="B3">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]=A3),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]=A3))</f>
-        <v>9990013.1860319264</v>
+      <c r="A3" s="4" t="e">
+        <f ca="1"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="B3" s="5" t="e" cm="1">
+        <f t="array" aca="1" ref="B3" ca="1">SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]=A3),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]=A3))</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>46101</v>
-      </c>
-      <c r="B4" s="5" cm="1">
-        <f t="array" ref="B4">B3+SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A4),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A4))</f>
-        <v>9990691.4268346932</v>
+      <c r="A4" s="4" t="e">
+        <f ca="1"/>
+        <v>#NAME?</v>
+      </c>
+      <c r="B4" s="5" t="e" cm="1">
+        <f t="array" aca="1" ref="B4" ca="1">B3+SUMPRODUCT(_xlfn._xlws.FILTER(Operaciones_table[Cantidad],Operaciones_table[Fecha]='Valor cartera'!A4),_xlfn._xlws.FILTER(Operaciones_table[Precio],Operaciones_table[Fecha]='Valor cartera'!A4))</f>
+        <v>#NAME?</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>46108</v>
+      <c r="A5" s="4" t="e">
+        <f ca="1"/>
+        <v>#NAME?</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
envío 10 de abril
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Master Quant\Gestión de activos\Trabajo gestión cuantitativa\Trabajo_gestion_cuantitativa\Trabajo_gestion_cuantitativa\Envíos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B4E8EB-8366-4071-B11E-B048FB6ABFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99C1D2B-03A9-4F8A-BBD5-F80953E30FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -229,10 +229,10 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="10" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
@@ -282,16 +282,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G74" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:G74" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G89" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:G89" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
     <tableColumn id="3" xr3:uid="{A21132F4-DD79-4C51-BEA4-4132F3EE35CB}" name="Acción"/>
     <tableColumn id="4" xr3:uid="{6F333961-151C-4394-89A0-8580A62F023E}" name="Cantidad"/>
     <tableColumn id="5" xr3:uid="{42F80897-162E-4CCE-9055-2FE010A8018C}" name="Precio" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{4564E466-B65B-45FE-ABC2-4D8C13865180}" name="CT" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{D63DF80C-BC33-4512-86ED-550CC24A9DC5}" name="Precio Ejecutado" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -520,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -568,7 +568,7 @@
       <c r="E2" s="2">
         <v>1</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G2" s="2">
@@ -593,7 +593,7 @@
       <c r="E3" s="2">
         <v>1180.40002441406</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G3" s="2">
@@ -618,7 +618,7 @@
       <c r="E4" s="2">
         <v>152.64999389648401</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G4" s="2">
@@ -643,7 +643,7 @@
       <c r="E5" s="2">
         <v>18.184999465942301</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G5" s="2">
@@ -668,7 +668,7 @@
       <c r="E6" s="2">
         <v>141.19999694824199</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G6" s="2">
@@ -693,7 +693,7 @@
       <c r="E7" s="2">
         <v>45.430000305175703</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G7" s="2">
@@ -718,7 +718,7 @@
       <c r="E8" s="2">
         <v>167.02000427246</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G8" s="2">
@@ -743,7 +743,7 @@
       <c r="E9" s="2">
         <v>210.80000305175699</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G9" s="2">
@@ -768,7 +768,7 @@
       <c r="E10" s="2">
         <v>292.600006103515</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G10" s="2">
@@ -793,7 +793,7 @@
       <c r="E11" s="2">
         <v>67.139999389648395</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G11" s="2">
@@ -818,7 +818,7 @@
       <c r="E12" s="2">
         <v>39.130001068115199</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G12" s="2">
@@ -843,7 +843,7 @@
       <c r="E13" s="2">
         <v>917.29998779296795</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G13" s="2">
@@ -868,7 +868,7 @@
       <c r="E14" s="2">
         <v>25.704999923706001</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G14" s="2">
@@ -893,7 +893,7 @@
       <c r="E15" s="2">
         <v>1550.5</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G15" s="2">
@@ -918,7 +918,7 @@
       <c r="E16" s="2">
         <v>616</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G16" s="2">
@@ -943,7 +943,7 @@
       <c r="E17" s="2">
         <v>172.03999328613199</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G17" s="2">
@@ -968,7 +968,7 @@
       <c r="E18" s="2">
         <v>5.0297000000000001</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G18" s="2">
@@ -993,7 +993,7 @@
       <c r="E19" s="2">
         <v>194.75</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G19" s="2">
@@ -1016,7 +1016,7 @@
       <c r="E20" s="2">
         <v>863.5</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G20" s="2">
@@ -1039,7 +1039,7 @@
       <c r="E21" s="2">
         <v>40.020000457763601</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G21" s="2">
@@ -1062,7 +1062,7 @@
       <c r="E22" s="2">
         <v>140.75</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F22">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G22" s="2">
@@ -1085,7 +1085,7 @@
       <c r="E23" s="2">
         <v>133.5</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G23" s="2">
@@ -1108,7 +1108,7 @@
       <c r="E24" s="2">
         <v>273.79998779296801</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F24">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G24" s="2">
@@ -1131,7 +1131,7 @@
       <c r="E25" s="2">
         <v>153.82000732421801</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F25">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G25" s="2">
@@ -1154,7 +1154,7 @@
       <c r="E26" s="2">
         <v>1656</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G26" s="2">
@@ -1177,7 +1177,7 @@
       <c r="E27" s="2">
         <v>23.620000839233398</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F27">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G27" s="2">
@@ -1200,7 +1200,7 @@
       <c r="E28" s="2">
         <v>68.080001831054602</v>
       </c>
-      <c r="F28" s="6">
+      <c r="F28">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G28" s="2">
@@ -1223,7 +1223,7 @@
       <c r="E29" s="2">
         <v>65.440002441406193</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F29">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G29" s="2">
@@ -1246,7 +1246,7 @@
       <c r="E30" s="2">
         <v>584.79998779296795</v>
       </c>
-      <c r="F30" s="6">
+      <c r="F30">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G30" s="2">
@@ -1270,7 +1270,7 @@
       <c r="E31" s="2">
         <v>38.384998321533203</v>
       </c>
-      <c r="F31" s="6">
+      <c r="F31">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G31" s="2">
@@ -1293,7 +1293,7 @@
       <c r="E32" s="2">
         <v>24.7600002288818</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F32">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G32" s="2">
@@ -1316,7 +1316,7 @@
       <c r="E33" s="2">
         <v>17.924999237060501</v>
       </c>
-      <c r="F33" s="6">
+      <c r="F33">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G33" s="2">
@@ -1339,7 +1339,7 @@
       <c r="E34" s="2">
         <v>1503</v>
       </c>
-      <c r="F34" s="6">
+      <c r="F34">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G34" s="2">
@@ -1362,7 +1362,7 @@
       <c r="E35" s="2">
         <v>1128.19995117187</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G35" s="2">
@@ -1385,7 +1385,7 @@
       <c r="E36" s="2">
         <v>160.919998168945</v>
       </c>
-      <c r="F36" s="6">
+      <c r="F36">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G36" s="2">
@@ -1408,7 +1408,7 @@
       <c r="E37" s="2">
         <v>37.430000305175703</v>
       </c>
-      <c r="F37" s="6">
+      <c r="F37">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G37" s="2">
@@ -1431,7 +1431,7 @@
       <c r="E38" s="2">
         <v>23.924999237060501</v>
       </c>
-      <c r="F38" s="6">
+      <c r="F38">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G38" s="2">
@@ -1454,7 +1454,7 @@
       <c r="E39" s="2">
         <v>1146.40002441406</v>
       </c>
-      <c r="F39" s="6">
+      <c r="F39">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G39" s="2">
@@ -1477,7 +1477,7 @@
       <c r="E40" s="2">
         <v>1379.5</v>
       </c>
-      <c r="F40" s="6">
+      <c r="F40">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G40" s="2">
@@ -1500,7 +1500,7 @@
       <c r="E41" s="2">
         <v>78.489997863769503</v>
       </c>
-      <c r="F41" s="6">
+      <c r="F41">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G41" s="2">
@@ -1523,7 +1523,7 @@
       <c r="E42" s="2">
         <v>60.220001220703097</v>
       </c>
-      <c r="F42" s="6">
+      <c r="F42">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G42" s="2">
@@ -1546,7 +1546,7 @@
       <c r="E43" s="2">
         <v>278.39999389648398</v>
       </c>
-      <c r="F43" s="6">
+      <c r="F43">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G43" s="2">
@@ -1569,7 +1569,7 @@
       <c r="E44" s="2">
         <v>21.7199993133544</v>
       </c>
-      <c r="F44" s="6">
+      <c r="F44">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G44" s="2">
@@ -1592,7 +1592,7 @@
       <c r="E45" s="2">
         <v>9.4020004272460902</v>
       </c>
-      <c r="F45" s="6">
+      <c r="F45">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G45" s="2">
@@ -1615,7 +1615,7 @@
       <c r="E46" s="2">
         <v>38.259998321533203</v>
       </c>
-      <c r="F46" s="6">
+      <c r="F46">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G46" s="2">
@@ -1638,7 +1638,7 @@
       <c r="E47" s="2">
         <v>69.120002746582003</v>
       </c>
-      <c r="F47" s="6">
+      <c r="F47">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G47" s="2">
@@ -1661,7 +1661,7 @@
       <c r="E48" s="2">
         <v>24.915000915527301</v>
       </c>
-      <c r="F48" s="6">
+      <c r="F48">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G48" s="2">
@@ -1684,7 +1684,7 @@
       <c r="E49" s="2">
         <v>132.05000305175699</v>
       </c>
-      <c r="F49" s="6">
+      <c r="F49">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G49" s="2">
@@ -1707,7 +1707,7 @@
       <c r="E50" s="2">
         <v>38.720001220703097</v>
       </c>
-      <c r="F50" s="6">
+      <c r="F50">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G50" s="2">
@@ -1730,7 +1730,7 @@
       <c r="E51" s="2">
         <v>194.80000305175699</v>
       </c>
-      <c r="F51" s="6">
+      <c r="F51">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G51" s="2">
@@ -1753,7 +1753,7 @@
       <c r="E52" s="2">
         <v>607.40002441406205</v>
       </c>
-      <c r="F52" s="6">
+      <c r="F52">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G52" s="2">
@@ -1776,7 +1776,7 @@
       <c r="E53" s="2">
         <v>1621.5</v>
       </c>
-      <c r="F53" s="6">
+      <c r="F53">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G53" s="2">
@@ -1799,7 +1799,7 @@
       <c r="E54" s="2">
         <v>62.319999694824197</v>
       </c>
-      <c r="F54" s="6">
+      <c r="F54">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G54" s="2">
@@ -1822,7 +1822,7 @@
       <c r="E55" s="2">
         <v>278.29998779296801</v>
       </c>
-      <c r="F55" s="6">
+      <c r="F55">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G55" s="2">
@@ -1845,7 +1845,7 @@
       <c r="E56" s="2">
         <v>142.55999755859301</v>
       </c>
-      <c r="F56" s="6">
+      <c r="F56">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G56" s="2">
@@ -1868,7 +1868,7 @@
       <c r="E57" s="2">
         <v>855.5</v>
       </c>
-      <c r="F57" s="6">
+      <c r="F57">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G57" s="2">
@@ -1891,7 +1891,7 @@
       <c r="E58" s="2">
         <v>144.39999389648401</v>
       </c>
-      <c r="F58" s="6">
+      <c r="F58">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G58" s="2">
@@ -1914,7 +1914,7 @@
       <c r="E59" s="2">
         <v>39.694999694824197</v>
       </c>
-      <c r="F59" s="6">
+      <c r="F59">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G59" s="2">
@@ -1937,7 +1937,7 @@
       <c r="E60" s="2">
         <v>18.770000457763601</v>
       </c>
-      <c r="F60" s="6">
+      <c r="F60">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G60" s="2">
@@ -1960,7 +1960,7 @@
       <c r="E61" s="2">
         <v>295.5</v>
       </c>
-      <c r="F61" s="6">
+      <c r="F61">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G61" s="2">
@@ -1983,7 +1983,7 @@
       <c r="E62" s="2">
         <v>287.29998779296801</v>
       </c>
-      <c r="F62" s="6">
+      <c r="F62">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G62" s="2">
@@ -2006,7 +2006,7 @@
       <c r="E63" s="2">
         <v>1161</v>
       </c>
-      <c r="F63" s="6">
+      <c r="F63">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G63" s="2">
@@ -2029,7 +2029,7 @@
       <c r="E64" s="2">
         <v>134.89999389648401</v>
       </c>
-      <c r="F64" s="6">
+      <c r="F64">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G64" s="2">
@@ -2052,7 +2052,7 @@
       <c r="E65" s="2">
         <v>25.674999237060501</v>
       </c>
-      <c r="F65" s="6">
+      <c r="F65">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G65" s="2">
@@ -2075,7 +2075,7 @@
       <c r="E66" s="2">
         <v>38.959999084472599</v>
       </c>
-      <c r="F66" s="6">
+      <c r="F66">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G66" s="2">
@@ -2098,7 +2098,7 @@
       <c r="E67" s="2">
         <v>79.419998168945298</v>
       </c>
-      <c r="F67" s="6">
+      <c r="F67">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G67" s="2">
@@ -2121,7 +2121,7 @@
       <c r="E68" s="2">
         <v>70.519996643066406</v>
       </c>
-      <c r="F68" s="6">
+      <c r="F68">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G68" s="2">
@@ -2144,7 +2144,7 @@
       <c r="E69" s="2">
         <v>149.69999694824199</v>
       </c>
-      <c r="F69" s="6">
+      <c r="F69">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G69" s="2">
@@ -2167,7 +2167,7 @@
       <c r="E70" s="2">
         <v>62.659999847412102</v>
       </c>
-      <c r="F70" s="6">
+      <c r="F70">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G70" s="2">
@@ -2190,7 +2190,7 @@
       <c r="E71" s="2">
         <v>22.944999694824201</v>
       </c>
-      <c r="F71" s="6">
+      <c r="F71">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G71" s="2">
@@ -2213,7 +2213,7 @@
       <c r="E72" s="2">
         <v>24.684999465942301</v>
       </c>
-      <c r="F72" s="6">
+      <c r="F72">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G72" s="2">
@@ -2236,7 +2236,7 @@
       <c r="E73" s="2">
         <v>1570.5</v>
       </c>
-      <c r="F73" s="6">
+      <c r="F73">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G73" s="2">
@@ -2259,11 +2259,356 @@
       <c r="E74" s="2">
         <v>9.8140001296996999</v>
       </c>
-      <c r="F74" s="6">
+      <c r="F74">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="G74" s="2">
         <v>9.8090931296348494</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B75" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" t="s">
+        <v>23</v>
+      </c>
+      <c r="D75">
+        <v>2584</v>
+      </c>
+      <c r="E75" s="2">
+        <v>41.555000305175703</v>
+      </c>
+      <c r="F75" s="6">
+        <v>2.0777500152587801E-2</v>
+      </c>
+      <c r="G75" s="2">
+        <v>41.5757778053283</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B76" t="s">
+        <v>37</v>
+      </c>
+      <c r="C76" t="s">
+        <v>23</v>
+      </c>
+      <c r="D76">
+        <v>19597</v>
+      </c>
+      <c r="E76" s="2">
+        <v>10.5159997940063</v>
+      </c>
+      <c r="F76" s="6">
+        <v>5.2579998970031698E-3</v>
+      </c>
+      <c r="G76" s="2">
+        <v>10.521257793903301</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B77" t="s">
+        <v>6</v>
+      </c>
+      <c r="C77" t="s">
+        <v>23</v>
+      </c>
+      <c r="D77">
+        <v>6951</v>
+      </c>
+      <c r="E77" s="2">
+        <v>167.22000122070301</v>
+      </c>
+      <c r="F77" s="6">
+        <v>8.3610000610351495E-2</v>
+      </c>
+      <c r="G77" s="2">
+        <v>167.30361122131299</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B78" t="s">
+        <v>16</v>
+      </c>
+      <c r="C78" t="s">
+        <v>23</v>
+      </c>
+      <c r="D78">
+        <v>663</v>
+      </c>
+      <c r="E78" s="2">
+        <v>27.709999084472599</v>
+      </c>
+      <c r="F78" s="6">
+        <v>1.3854999542236301E-2</v>
+      </c>
+      <c r="G78" s="2">
+        <v>27.7238540840148</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B79" t="s">
+        <v>8</v>
+      </c>
+      <c r="C79" t="s">
+        <v>23</v>
+      </c>
+      <c r="D79">
+        <v>1900</v>
+      </c>
+      <c r="E79" s="2">
+        <v>137.80000305175699</v>
+      </c>
+      <c r="F79" s="6">
+        <v>6.8900001525878898E-2</v>
+      </c>
+      <c r="G79" s="2">
+        <v>137.86890305328299</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B80" t="s">
+        <v>33</v>
+      </c>
+      <c r="C80" t="s">
+        <v>23</v>
+      </c>
+      <c r="D80">
+        <v>3599</v>
+      </c>
+      <c r="E80" s="2">
+        <v>78.610000610351506</v>
+      </c>
+      <c r="F80" s="6">
+        <v>3.9305000305175697E-2</v>
+      </c>
+      <c r="G80" s="2">
+        <v>78.649305610656697</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B81" t="s">
+        <v>14</v>
+      </c>
+      <c r="C81" t="s">
+        <v>23</v>
+      </c>
+      <c r="D81">
+        <v>5804</v>
+      </c>
+      <c r="E81" s="2">
+        <v>40.119998931884702</v>
+      </c>
+      <c r="F81" s="6">
+        <v>2.0059999465942301E-2</v>
+      </c>
+      <c r="G81" s="2">
+        <v>40.140058931350701</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B82" t="s">
+        <v>25</v>
+      </c>
+      <c r="C82" t="s">
+        <v>26</v>
+      </c>
+      <c r="D82">
+        <v>-3328</v>
+      </c>
+      <c r="E82" s="2">
+        <v>23.9500007629394</v>
+      </c>
+      <c r="F82" s="6">
+        <v>1.1975000381469701E-2</v>
+      </c>
+      <c r="G82" s="2">
+        <v>23.938025762557899</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B83" t="s">
+        <v>7</v>
+      </c>
+      <c r="C83" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83">
+        <v>-36557</v>
+      </c>
+      <c r="E83" s="2">
+        <v>19.704999923706001</v>
+      </c>
+      <c r="F83" s="6">
+        <v>9.8524999618530198E-3</v>
+      </c>
+      <c r="G83" s="2">
+        <v>19.695147423744199</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B84" t="s">
+        <v>35</v>
+      </c>
+      <c r="C84" t="s">
+        <v>26</v>
+      </c>
+      <c r="D84">
+        <v>-400</v>
+      </c>
+      <c r="E84" s="2">
+        <v>313.29998779296801</v>
+      </c>
+      <c r="F84" s="6">
+        <v>0.15664999389648401</v>
+      </c>
+      <c r="G84" s="2">
+        <v>313.14333779907201</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B85" t="s">
+        <v>15</v>
+      </c>
+      <c r="C85" t="s">
+        <v>26</v>
+      </c>
+      <c r="D85">
+        <v>-294</v>
+      </c>
+      <c r="E85" s="2">
+        <v>858.79998779296795</v>
+      </c>
+      <c r="F85" s="6">
+        <v>0.42939999389648398</v>
+      </c>
+      <c r="G85" s="2">
+        <v>858.37058779907204</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B86" t="s">
+        <v>28</v>
+      </c>
+      <c r="C86" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86">
+        <v>-3049</v>
+      </c>
+      <c r="E86" s="2">
+        <v>76</v>
+      </c>
+      <c r="F86" s="6">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="G86" s="2">
+        <v>75.962000000000003</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B87" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87">
+        <v>-569</v>
+      </c>
+      <c r="E87" s="2">
+        <v>1270</v>
+      </c>
+      <c r="F87" s="6">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="G87" s="2">
+        <v>1269.365</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B88" t="s">
+        <v>32</v>
+      </c>
+      <c r="C88" t="s">
+        <v>26</v>
+      </c>
+      <c r="D88">
+        <v>-2481</v>
+      </c>
+      <c r="E88" s="2">
+        <v>42.825000762939403</v>
+      </c>
+      <c r="F88" s="6">
+        <v>2.1412500381469701E-2</v>
+      </c>
+      <c r="G88" s="2">
+        <v>42.803588262557902</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" s="4">
+        <v>46122</v>
+      </c>
+      <c r="B89" t="s">
+        <v>12</v>
+      </c>
+      <c r="C89" t="s">
+        <v>26</v>
+      </c>
+      <c r="D89">
+        <v>-115</v>
+      </c>
+      <c r="E89" s="2">
+        <v>301.64999389648398</v>
+      </c>
+      <c r="F89" s="6">
+        <v>0.150824996948242</v>
+      </c>
+      <c r="G89" s="2">
+        <v>301.49916889953602</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
envío 17 de abril
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Master Quant\Gestión de activos\Trabajo gestión cuantitativa\Trabajo_gestion_cuantitativa\Trabajo_gestion_cuantitativa\Envíos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D99C1D2B-03A9-4F8A-BBD5-F80953E30FDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A599AE5F-EC26-4E6F-B9B5-628D0FE8F665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="39">
   <si>
     <t>ID</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>SAN.MC</t>
+  </si>
+  <si>
+    <t>ITX.MC</t>
   </si>
 </sst>
 </file>
@@ -282,8 +285,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G89" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:G89" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:G107" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:G107" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
@@ -520,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -2282,7 +2285,7 @@
       <c r="E75" s="2">
         <v>41.555000305175703</v>
       </c>
-      <c r="F75" s="6">
+      <c r="F75">
         <v>2.0777500152587801E-2</v>
       </c>
       <c r="G75" s="2">
@@ -2305,7 +2308,7 @@
       <c r="E76" s="2">
         <v>10.5159997940063</v>
       </c>
-      <c r="F76" s="6">
+      <c r="F76">
         <v>5.2579998970031698E-3</v>
       </c>
       <c r="G76" s="2">
@@ -2328,7 +2331,7 @@
       <c r="E77" s="2">
         <v>167.22000122070301</v>
       </c>
-      <c r="F77" s="6">
+      <c r="F77">
         <v>8.3610000610351495E-2</v>
       </c>
       <c r="G77" s="2">
@@ -2351,7 +2354,7 @@
       <c r="E78" s="2">
         <v>27.709999084472599</v>
       </c>
-      <c r="F78" s="6">
+      <c r="F78">
         <v>1.3854999542236301E-2</v>
       </c>
       <c r="G78" s="2">
@@ -2374,7 +2377,7 @@
       <c r="E79" s="2">
         <v>137.80000305175699</v>
       </c>
-      <c r="F79" s="6">
+      <c r="F79">
         <v>6.8900001525878898E-2</v>
       </c>
       <c r="G79" s="2">
@@ -2397,7 +2400,7 @@
       <c r="E80" s="2">
         <v>78.610000610351506</v>
       </c>
-      <c r="F80" s="6">
+      <c r="F80">
         <v>3.9305000305175697E-2</v>
       </c>
       <c r="G80" s="2">
@@ -2420,7 +2423,7 @@
       <c r="E81" s="2">
         <v>40.119998931884702</v>
       </c>
-      <c r="F81" s="6">
+      <c r="F81">
         <v>2.0059999465942301E-2</v>
       </c>
       <c r="G81" s="2">
@@ -2443,7 +2446,7 @@
       <c r="E82" s="2">
         <v>23.9500007629394</v>
       </c>
-      <c r="F82" s="6">
+      <c r="F82">
         <v>1.1975000381469701E-2</v>
       </c>
       <c r="G82" s="2">
@@ -2466,7 +2469,7 @@
       <c r="E83" s="2">
         <v>19.704999923706001</v>
       </c>
-      <c r="F83" s="6">
+      <c r="F83">
         <v>9.8524999618530198E-3</v>
       </c>
       <c r="G83" s="2">
@@ -2489,7 +2492,7 @@
       <c r="E84" s="2">
         <v>313.29998779296801</v>
       </c>
-      <c r="F84" s="6">
+      <c r="F84">
         <v>0.15664999389648401</v>
       </c>
       <c r="G84" s="2">
@@ -2512,7 +2515,7 @@
       <c r="E85" s="2">
         <v>858.79998779296795</v>
       </c>
-      <c r="F85" s="6">
+      <c r="F85">
         <v>0.42939999389648398</v>
       </c>
       <c r="G85" s="2">
@@ -2535,7 +2538,7 @@
       <c r="E86" s="2">
         <v>76</v>
       </c>
-      <c r="F86" s="6">
+      <c r="F86">
         <v>3.7999999999999999E-2</v>
       </c>
       <c r="G86" s="2">
@@ -2558,7 +2561,7 @@
       <c r="E87" s="2">
         <v>1270</v>
       </c>
-      <c r="F87" s="6">
+      <c r="F87">
         <v>0.63500000000000001</v>
       </c>
       <c r="G87" s="2">
@@ -2581,7 +2584,7 @@
       <c r="E88" s="2">
         <v>42.825000762939403</v>
       </c>
-      <c r="F88" s="6">
+      <c r="F88">
         <v>2.1412500381469701E-2</v>
       </c>
       <c r="G88" s="2">
@@ -2604,11 +2607,425 @@
       <c r="E89" s="2">
         <v>301.64999389648398</v>
       </c>
-      <c r="F89" s="6">
+      <c r="F89">
         <v>0.150824996948242</v>
       </c>
       <c r="G89" s="2">
         <v>301.49916889953602</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B90" t="s">
+        <v>33</v>
+      </c>
+      <c r="C90" t="s">
+        <v>23</v>
+      </c>
+      <c r="D90">
+        <v>2329</v>
+      </c>
+      <c r="E90" s="2">
+        <v>73.069999694824205</v>
+      </c>
+      <c r="F90" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G90" s="2">
+        <v>73.106534694671595</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B91" t="s">
+        <v>16</v>
+      </c>
+      <c r="C91" t="s">
+        <v>23</v>
+      </c>
+      <c r="D91">
+        <v>6891</v>
+      </c>
+      <c r="E91" s="2">
+        <v>28.909999847412099</v>
+      </c>
+      <c r="F91" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G91" s="2">
+        <v>28.924454847335799</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B92" t="s">
+        <v>13</v>
+      </c>
+      <c r="C92" t="s">
+        <v>23</v>
+      </c>
+      <c r="D92">
+        <v>3946</v>
+      </c>
+      <c r="E92" s="2">
+        <v>71.339996337890597</v>
+      </c>
+      <c r="F92" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G92" s="2">
+        <v>71.375666336059496</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B93" t="s">
+        <v>38</v>
+      </c>
+      <c r="C93" t="s">
+        <v>23</v>
+      </c>
+      <c r="D93">
+        <v>4327</v>
+      </c>
+      <c r="E93" s="2">
+        <v>55.020000457763601</v>
+      </c>
+      <c r="F93" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G93" s="2">
+        <v>55.047510457992502</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B94" t="s">
+        <v>10</v>
+      </c>
+      <c r="C94" t="s">
+        <v>23</v>
+      </c>
+      <c r="D94">
+        <v>1388</v>
+      </c>
+      <c r="E94" s="2">
+        <v>156.24000549316401</v>
+      </c>
+      <c r="F94" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G94" s="2">
+        <v>156.31812549591001</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B95" t="s">
+        <v>14</v>
+      </c>
+      <c r="C95" t="s">
+        <v>23</v>
+      </c>
+      <c r="D95">
+        <v>19134</v>
+      </c>
+      <c r="E95" s="2">
+        <v>41.099998474121001</v>
+      </c>
+      <c r="F95" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G95" s="2">
+        <v>41.120548473358099</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B96" t="s">
+        <v>7</v>
+      </c>
+      <c r="C96" t="s">
+        <v>23</v>
+      </c>
+      <c r="D96">
+        <v>832</v>
+      </c>
+      <c r="E96" s="2">
+        <v>20.309999465942301</v>
+      </c>
+      <c r="F96" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G96" s="2">
+        <v>20.320154465675301</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B97" t="s">
+        <v>5</v>
+      </c>
+      <c r="C97" t="s">
+        <v>23</v>
+      </c>
+      <c r="D97">
+        <v>674</v>
+      </c>
+      <c r="E97" s="2">
+        <v>1244</v>
+      </c>
+      <c r="F97" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G97" s="2">
+        <v>1244.6219999999901</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B98" t="s">
+        <v>28</v>
+      </c>
+      <c r="C98" t="s">
+        <v>26</v>
+      </c>
+      <c r="D98">
+        <v>674</v>
+      </c>
+      <c r="E98" s="2">
+        <v>81.440002441406193</v>
+      </c>
+      <c r="F98" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G98" s="2">
+        <v>81.399282440185502</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B99" t="s">
+        <v>15</v>
+      </c>
+      <c r="C99" t="s">
+        <v>26</v>
+      </c>
+      <c r="D99">
+        <v>-81</v>
+      </c>
+      <c r="E99" s="2">
+        <v>984.90002441406205</v>
+      </c>
+      <c r="F99" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G99" s="2">
+        <v>984.40757440185496</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B100" t="s">
+        <v>9</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100">
+        <v>-803</v>
+      </c>
+      <c r="E100" s="2">
+        <v>44.330001831054602</v>
+      </c>
+      <c r="F100" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G100" s="2">
+        <v>44.307836830139102</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B101" t="s">
+        <v>32</v>
+      </c>
+      <c r="C101" t="s">
+        <v>26</v>
+      </c>
+      <c r="D101">
+        <v>-6028</v>
+      </c>
+      <c r="E101" s="2">
+        <v>48.900001525878899</v>
+      </c>
+      <c r="F101" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G101" s="2">
+        <v>48.875551525115903</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B102" t="s">
+        <v>25</v>
+      </c>
+      <c r="C102" t="s">
+        <v>26</v>
+      </c>
+      <c r="D102">
+        <v>-938</v>
+      </c>
+      <c r="E102" s="2">
+        <v>21.7600002288818</v>
+      </c>
+      <c r="F102" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G102" s="2">
+        <v>21.7491202287673</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B103" t="s">
+        <v>6</v>
+      </c>
+      <c r="C103" t="s">
+        <v>26</v>
+      </c>
+      <c r="D103">
+        <v>-4228</v>
+      </c>
+      <c r="E103" s="2">
+        <v>172.05999755859301</v>
+      </c>
+      <c r="F103" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G103" s="2">
+        <v>171.97396755981401</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B104" t="s">
+        <v>37</v>
+      </c>
+      <c r="C104" t="s">
+        <v>26</v>
+      </c>
+      <c r="D104">
+        <v>-50484</v>
+      </c>
+      <c r="E104" s="2">
+        <v>11.041999816894499</v>
+      </c>
+      <c r="F104" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G104" s="2">
+        <v>11.036478816986</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B105" t="s">
+        <v>12</v>
+      </c>
+      <c r="C105" t="s">
+        <v>26</v>
+      </c>
+      <c r="D105">
+        <v>-1010</v>
+      </c>
+      <c r="E105" s="2">
+        <v>321.100006103515</v>
+      </c>
+      <c r="F105" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G105" s="2">
+        <v>320.93945610046302</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B106" t="s">
+        <v>35</v>
+      </c>
+      <c r="C106" t="s">
+        <v>26</v>
+      </c>
+      <c r="D106">
+        <v>-1147</v>
+      </c>
+      <c r="E106" s="2">
+        <v>315.29998779296801</v>
+      </c>
+      <c r="F106" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G106" s="2">
+        <v>315.14233779907198</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" s="4">
+        <v>46129</v>
+      </c>
+      <c r="B107" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107" t="s">
+        <v>26</v>
+      </c>
+      <c r="D107">
+        <v>-1401</v>
+      </c>
+      <c r="E107" s="2">
+        <v>146.39999389648401</v>
+      </c>
+      <c r="F107" s="6">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G107" s="2">
+        <v>146.326793899536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Envío 1 de mayo 2026
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Master Quant\Gestión de activos\Trabajo gestión cuantitativa\Trabajo_gestion_cuantitativa\Trabajo_gestion_cuantitativa\Envíos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC62BF2A-D9D1-4473-98F9-BF39A6C968A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FB0ABF-1B28-413B-A3EC-18775D89F40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
     <sheet name="Valor cartera" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" calcOnSave="0"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId3"/>
+    <pivotCache cacheId="43" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -187,6 +187,15 @@
   <si>
     <t>Precio total</t>
   </si>
+  <si>
+    <t>BNP.PA</t>
+  </si>
+  <si>
+    <t>Cash de cada operación (&gt;0 si vendemos más que compramos, &lt;0 en caso contrario)</t>
+  </si>
+  <si>
+    <t>Posiciones compradas o vendidas por fecha y activo</t>
+  </si>
 </sst>
 </file>
 
@@ -196,7 +205,7 @@
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -210,6 +219,14 @@
       <color theme="0"/>
       <name val="Amasis MT Pro"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Amasis MT Pro"/>
+      <family val="1"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -239,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -250,6 +267,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="6" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -313,13 +332,13 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="estadio gijon" refreshedDate="46140.5098119213" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="123" xr:uid="{F974E3A8-FD59-40A3-ACE6-0C536987A82A}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="estadio gijon" refreshedDate="46143.824766203703" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="145" xr:uid="{F974E3A8-FD59-40A3-ACE6-0C536987A82A}">
   <cacheSource type="worksheet">
     <worksheetSource name="Operaciones_table"/>
   </cacheSource>
   <cacheFields count="10">
     <cacheField name="Fecha" numFmtId="14">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-03-11T00:00:00" maxDate="2026-04-25T00:00:00" count="8">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-03-11T00:00:00" maxDate="2026-05-23T00:00:00" count="30">
         <d v="2026-03-11T00:00:00"/>
         <d v="2026-03-12T00:00:00"/>
         <d v="2026-03-20T00:00:00"/>
@@ -328,11 +347,33 @@
         <d v="2026-04-10T00:00:00"/>
         <d v="2026-04-17T00:00:00"/>
         <d v="2026-04-24T00:00:00"/>
+        <d v="2026-05-01T00:00:00"/>
+        <d v="2026-05-02T00:00:00" u="1"/>
+        <d v="2026-05-03T00:00:00" u="1"/>
+        <d v="2026-05-04T00:00:00" u="1"/>
+        <d v="2026-05-05T00:00:00" u="1"/>
+        <d v="2026-05-06T00:00:00" u="1"/>
+        <d v="2026-05-07T00:00:00" u="1"/>
+        <d v="2026-05-08T00:00:00" u="1"/>
+        <d v="2026-05-09T00:00:00" u="1"/>
+        <d v="2026-05-10T00:00:00" u="1"/>
+        <d v="2026-05-11T00:00:00" u="1"/>
+        <d v="2026-05-12T00:00:00" u="1"/>
+        <d v="2026-05-13T00:00:00" u="1"/>
+        <d v="2026-05-14T00:00:00" u="1"/>
+        <d v="2026-05-15T00:00:00" u="1"/>
+        <d v="2026-05-16T00:00:00" u="1"/>
+        <d v="2026-05-17T00:00:00" u="1"/>
+        <d v="2026-05-18T00:00:00" u="1"/>
+        <d v="2026-05-19T00:00:00" u="1"/>
+        <d v="2026-05-20T00:00:00" u="1"/>
+        <d v="2026-05-21T00:00:00" u="1"/>
+        <d v="2026-05-22T00:00:00" u="1"/>
       </sharedItems>
       <fieldGroup par="9"/>
     </cacheField>
     <cacheField name="ID" numFmtId="0">
-      <sharedItems count="27">
+      <sharedItems count="28">
         <s v="CASH"/>
         <s v="ASML.AS"/>
         <s v="ENR.DE"/>
@@ -360,6 +401,7 @@
         <s v="INGA.AS"/>
         <s v="SAN.MC"/>
         <s v="ITX.MC"/>
+        <s v="BNP.PA"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Acción" numFmtId="0">
@@ -372,7 +414,7 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1" maxValue="1656"/>
     </cacheField>
     <cacheField name="CT" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.0000000000000001E-4" maxValue="0.65959997558593697"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.0000000000000001E-4" maxValue="5.0000000000000001E-4"/>
     </cacheField>
     <cacheField name="Precio Ejecutado" numFmtId="6">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1" maxValue="1656.828"/>
@@ -382,7 +424,7 @@
     </cacheField>
     <cacheField name="Days (Fecha)" numFmtId="0" databaseField="0">
       <fieldGroup base="0">
-        <rangePr groupBy="days" startDate="2026-03-11T00:00:00" endDate="2026-04-25T00:00:00"/>
+        <rangePr groupBy="days" startDate="2026-03-11T00:00:00" endDate="2026-05-02T00:00:00"/>
         <groupItems count="368">
           <s v="&lt;11/03/2026"/>
           <s v="01-ene"/>
@@ -751,13 +793,13 @@
           <s v="29-dic"/>
           <s v="30-dic"/>
           <s v="31-dic"/>
-          <s v="&gt;25/04/2026"/>
+          <s v="&gt;02/05/2026"/>
         </groupItems>
       </fieldGroup>
     </cacheField>
     <cacheField name="Months (Fecha)" numFmtId="0" databaseField="0">
       <fieldGroup base="0">
-        <rangePr groupBy="months" startDate="2026-03-11T00:00:00" endDate="2026-04-25T00:00:00"/>
+        <rangePr groupBy="months" startDate="2026-03-11T00:00:00" endDate="2026-05-02T00:00:00"/>
         <groupItems count="14">
           <s v="&lt;11/03/2026"/>
           <s v="ene"/>
@@ -772,7 +814,7 @@
           <s v="oct"/>
           <s v="nov"/>
           <s v="dic"/>
-          <s v="&gt;25/04/2026"/>
+          <s v="&gt;02/05/2026"/>
         </groupItems>
       </fieldGroup>
     </cacheField>
@@ -786,7 +828,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="123">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="145">
   <r>
     <x v="0"/>
     <x v="0"/>
@@ -1523,7 +1565,7 @@
     <s v="COMPRA"/>
     <n v="2584"/>
     <n v="41.555000305175703"/>
-    <n v="2.0777500152587801E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="41.5757778053283"/>
     <n v="-107431.80984896833"/>
   </r>
@@ -1533,7 +1575,7 @@
     <s v="COMPRA"/>
     <n v="19597"/>
     <n v="10.5159997940063"/>
-    <n v="5.2579998970031698E-3"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="10.521257793903301"/>
     <n v="-206185.08898712299"/>
   </r>
@@ -1543,7 +1585,7 @@
     <s v="COMPRA"/>
     <n v="6951"/>
     <n v="167.22000122070301"/>
-    <n v="8.3610000610351495E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="167.30361122131299"/>
     <n v="-1162927.4015993467"/>
   </r>
@@ -1553,7 +1595,7 @@
     <s v="COMPRA"/>
     <n v="663"/>
     <n v="27.709999084472599"/>
-    <n v="1.3854999542236301E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="27.7238540840148"/>
     <n v="-18380.915257701814"/>
   </r>
@@ -1563,7 +1605,7 @@
     <s v="COMPRA"/>
     <n v="1900"/>
     <n v="137.80000305175699"/>
-    <n v="6.8900001525878898E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="137.86890305328299"/>
     <n v="-261950.91580123769"/>
   </r>
@@ -1573,7 +1615,7 @@
     <s v="COMPRA"/>
     <n v="3599"/>
     <n v="78.610000610351506"/>
-    <n v="3.9305000305175697E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="78.649305610656697"/>
     <n v="-283058.85089275346"/>
   </r>
@@ -1583,7 +1625,7 @@
     <s v="COMPRA"/>
     <n v="5804"/>
     <n v="40.119998931884702"/>
-    <n v="2.0059999465942301E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="40.140058931350701"/>
     <n v="-232972.90203755946"/>
   </r>
@@ -1593,7 +1635,7 @@
     <s v="VENTA"/>
     <n v="-3328"/>
     <n v="23.9500007629394"/>
-    <n v="1.1975000381469701E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="23.938025762557899"/>
     <n v="79665.749737792692"/>
   </r>
@@ -1603,7 +1645,7 @@
     <s v="VENTA"/>
     <n v="-36557"/>
     <n v="19.704999923706001"/>
-    <n v="9.8524999618530198E-3"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="19.695147423744199"/>
     <n v="719995.50436981674"/>
   </r>
@@ -1613,7 +1655,7 @@
     <s v="VENTA"/>
     <n v="-400"/>
     <n v="313.29998779296801"/>
-    <n v="0.15664999389648401"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="313.14333779907201"/>
     <n v="125257.33511962881"/>
   </r>
@@ -1623,7 +1665,7 @@
     <s v="VENTA"/>
     <n v="-294"/>
     <n v="858.79998779296795"/>
-    <n v="0.42939999389648398"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="858.37058779907204"/>
     <n v="252360.95281292719"/>
   </r>
@@ -1633,7 +1675,7 @@
     <s v="VENTA"/>
     <n v="-3049"/>
     <n v="76"/>
-    <n v="3.7999999999999999E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="75.962000000000003"/>
     <n v="231608.13800000001"/>
   </r>
@@ -1643,7 +1685,7 @@
     <s v="VENTA"/>
     <n v="-569"/>
     <n v="1270"/>
-    <n v="0.63500000000000001"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="1269.365"/>
     <n v="722268.68500000006"/>
   </r>
@@ -1653,7 +1695,7 @@
     <s v="VENTA"/>
     <n v="-2481"/>
     <n v="42.825000762939403"/>
-    <n v="2.1412500381469701E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="42.803588262557902"/>
     <n v="106195.70247940616"/>
   </r>
@@ -1663,7 +1705,7 @@
     <s v="VENTA"/>
     <n v="-115"/>
     <n v="301.64999389648398"/>
-    <n v="0.150824996948242"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="301.49916889953602"/>
     <n v="34672.404423446642"/>
   </r>
@@ -1853,7 +1895,7 @@
     <s v="COMPRA"/>
     <n v="2251"/>
     <n v="41.534999847412102"/>
-    <n v="2.0767499923705999E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="41.555767347335802"/>
     <n v="-93542.032298852893"/>
   </r>
@@ -1863,7 +1905,7 @@
     <s v="COMPRA"/>
     <n v="10225"/>
     <n v="22.9500007629394"/>
-    <n v="1.14750003814697E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="22.961475763320902"/>
     <n v="-234781.08967995623"/>
   </r>
@@ -1873,7 +1915,7 @@
     <s v="COMPRA"/>
     <n v="9644"/>
     <n v="18.579999923706001"/>
-    <n v="9.2899999618530193E-3"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="18.589289923667899"/>
     <n v="-179275.1120238532"/>
   </r>
@@ -1883,7 +1925,7 @@
     <s v="COMPRA"/>
     <n v="208"/>
     <n v="147.27999877929599"/>
-    <n v="7.3639999389648395E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="147.35363877868599"/>
     <n v="-30649.556865966686"/>
   </r>
@@ -1893,7 +1935,7 @@
     <s v="COMPRA"/>
     <n v="23473"/>
     <n v="52.560001373291001"/>
-    <n v="2.6280000686645499E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="52.586281373977599"/>
     <n v="-1234357.7826913763"/>
   </r>
@@ -1903,7 +1945,7 @@
     <s v="COMPRA"/>
     <n v="1059"/>
     <n v="66.419998168945298"/>
-    <n v="3.32099990844726E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="66.453208168029704"/>
     <n v="-70373.947449943458"/>
   </r>
@@ -1913,7 +1955,7 @@
     <s v="COMPRA"/>
     <n v="175"/>
     <n v="975.09997558593705"/>
-    <n v="0.48754998779296799"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="975.58752557372998"/>
     <n v="-170727.81697540273"/>
   </r>
@@ -1923,7 +1965,7 @@
     <s v="COMPRA"/>
     <n v="225"/>
     <n v="1319.19995117187"/>
-    <n v="0.65959997558593697"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="1319.85955114746"/>
     <n v="-296968.3990081785"/>
   </r>
@@ -1933,7 +1975,7 @@
     <s v="COMPRA"/>
     <n v="11124"/>
     <n v="54.150001525878899"/>
-    <n v="2.7075000762939401E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="54.177076526641798"/>
     <n v="-602665.79928236338"/>
   </r>
@@ -1943,7 +1985,7 @@
     <s v="COMPRA"/>
     <n v="3623"/>
     <n v="187.61999511718699"/>
-    <n v="9.3809997558593705E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="187.71380511474601"/>
     <n v="-680087.11593072477"/>
   </r>
@@ -1953,7 +1995,7 @@
     <s v="VENTA"/>
     <n v="-1055"/>
     <n v="77.540000915527301"/>
-    <n v="3.8770000457763597E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="77.501230915069499"/>
     <n v="81763.798615398322"/>
   </r>
@@ -1963,7 +2005,7 @@
     <s v="VENTA"/>
     <n v="-111"/>
     <n v="1249.59997558593"/>
-    <n v="0.62479998779296797"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="1248.9751755981399"/>
     <n v="138636.24449139353"/>
   </r>
@@ -1973,7 +2015,7 @@
     <s v="VENTA"/>
     <n v="-577"/>
     <n v="136.25"/>
-    <n v="6.8125000000000005E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="136.18187499999999"/>
     <n v="78576.94187499999"/>
   </r>
@@ -1983,7 +2025,7 @@
     <s v="VENTA"/>
     <n v="-27490"/>
     <n v="38.5"/>
-    <n v="1.925E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="38.48075"/>
     <n v="1057835.8175000001"/>
   </r>
@@ -1993,7 +2035,7 @@
     <s v="VENTA"/>
     <n v="-7468"/>
     <n v="27.059999465942301"/>
-    <n v="1.35299997329711E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="27.046469466209398"/>
     <n v="201983.03397365179"/>
   </r>
@@ -2003,7 +2045,7 @@
     <s v="VENTA"/>
     <n v="-1247"/>
     <n v="270"/>
-    <n v="0.13500000000000001"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="269.86500000000001"/>
     <n v="336521.65500000003"/>
   </r>
@@ -2013,19 +2055,239 @@
     <s v="VENTA"/>
     <n v="-22074"/>
     <n v="77"/>
-    <n v="3.85E-2"/>
+    <n v="5.0000000000000001E-4"/>
     <n v="76.961500000000001"/>
     <n v="1698848.1510000001"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="19"/>
+    <s v="COMPRA"/>
+    <n v="2037"/>
+    <n v="77.639999000000003"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="77.678818999499995"/>
+    <n v="-158231.75430198148"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="8"/>
+    <s v="COMPRA"/>
+    <n v="343"/>
+    <n v="293.35000600000001"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="293.49668100299999"/>
+    <n v="-100669.361584029"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="23"/>
+    <s v="COMPRA"/>
+    <n v="824"/>
+    <n v="273"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="273.13650000000001"/>
+    <n v="-225064.47600000002"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="12"/>
+    <s v="COMPRA"/>
+    <n v="11411"/>
+    <n v="26.5"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="26.513249999999999"/>
+    <n v="-302542.69575000001"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="25"/>
+    <s v="COMPRA"/>
+    <n v="14533"/>
+    <n v="10.3800001144409"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="10.3851901144981"/>
+    <n v="-150927.96793400089"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="17"/>
+    <s v="COMPRA"/>
+    <n v="130"/>
+    <n v="1623.5"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="1624.3117499999901"/>
+    <n v="-211160.52749999872"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="27"/>
+    <s v="COMPRA"/>
+    <n v="4104"/>
+    <n v="89.230003356933594"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="89.274618358612003"/>
+    <n v="-366383.03374374367"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="2"/>
+    <s v="COMPRA"/>
+    <n v="380"/>
+    <n v="180.58000183105401"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="180.67029183196999"/>
+    <n v="-68654.710896148594"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="5"/>
+    <s v="COMPRA"/>
+    <n v="1204"/>
+    <n v="41.069999694824197"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="41.090534694671597"/>
+    <n v="-49473.003772384604"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="18"/>
+    <s v="COMPRA"/>
+    <n v="9077"/>
+    <n v="24"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="24.012"/>
+    <n v="-217956.924"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="10"/>
+    <s v="COMPRA"/>
+    <n v="15813"/>
+    <n v="38.049999237060497"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="38.069024236678999"/>
+    <n v="-601985.48025460506"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="11"/>
+    <s v="COMPRA"/>
+    <n v="147"/>
+    <n v="958.5"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="958.97924999999998"/>
+    <n v="-140969.94975"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="1"/>
+    <s v="COMPRA"/>
+    <n v="101"/>
+    <n v="1222.40002441406"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="1223.01122442626"/>
+    <n v="-123524.13366705226"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="3"/>
+    <s v="COMPRA"/>
+    <n v="26551"/>
+    <n v="18.809999465942301"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="18.819404465675301"/>
+    <n v="-499674.00796814496"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="9"/>
+    <s v="VENTA"/>
+    <n v="-1215"/>
+    <n v="66.419998168945298"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="66.386788169860793"/>
+    <n v="80659.947626380861"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="6"/>
+    <s v="VENTA"/>
+    <n v="-96"/>
+    <n v="145.5"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="145.42724999999999"/>
+    <n v="13961.016"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="21"/>
+    <s v="VENTA"/>
+    <n v="-4731"/>
+    <n v="79.290000915527301"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="79.250355915069505"/>
+    <n v="374933.43383419386"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="24"/>
+    <s v="VENTA"/>
+    <n v="-28804"/>
+    <n v="24.754999160766602"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="24.742621661186199"/>
+    <n v="712686.47432880732"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="4"/>
+    <s v="VENTA"/>
+    <n v="-2741"/>
+    <n v="147.39999389648401"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="147.32629389953601"/>
+    <n v="403821.3715786282"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="26"/>
+    <s v="VENTA"/>
+    <n v="-27800"/>
+    <n v="50.580001831054602"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="50.554711830139098"/>
+    <n v="1405420.9888778669"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="13"/>
+    <s v="VENTA"/>
+    <n v="-7"/>
+    <n v="1355.80004882812"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="1355.1221488037099"/>
+    <n v="9485.8550416259695"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="20"/>
+    <s v="VENTA"/>
+    <n v="-3779"/>
+    <n v="57.130001068115199"/>
+    <n v="5.0000000000000001E-4"/>
+    <n v="57.101436067581098"/>
+    <n v="215786.32689938898"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA75CCB5-861C-4E63-A423-1C9A4AC3CFAA}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="J17:K26" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA75CCB5-861C-4E63-A423-1C9A4AC3CFAA}" name="PivotTable2" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="J3:K13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" numFmtId="14" showAll="0">
-      <items count="9">
+      <items count="31">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -2034,6 +2296,28 @@
         <item x="5"/>
         <item x="6"/>
         <item x="7"/>
+        <item x="8"/>
+        <item m="1" x="9"/>
+        <item m="1" x="10"/>
+        <item m="1" x="11"/>
+        <item m="1" x="12"/>
+        <item m="1" x="13"/>
+        <item m="1" x="14"/>
+        <item m="1" x="15"/>
+        <item m="1" x="16"/>
+        <item m="1" x="17"/>
+        <item m="1" x="18"/>
+        <item m="1" x="19"/>
+        <item m="1" x="20"/>
+        <item m="1" x="21"/>
+        <item m="1" x="22"/>
+        <item m="1" x="23"/>
+        <item m="1" x="24"/>
+        <item m="1" x="25"/>
+        <item m="1" x="26"/>
+        <item m="1" x="27"/>
+        <item m="1" x="28"/>
+        <item m="1" x="29"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -2440,7 +2724,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="9">
+  <rowItems count="10">
     <i>
       <x/>
     </i>
@@ -2465,6 +2749,9 @@
     <i>
       <x v="7"/>
     </i>
+    <i>
+      <x v="8"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
@@ -2488,11 +2775,11 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98EFF2E4-313D-4FF3-8D4A-C66D4400DAC9}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="J3:L11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98EFF2E4-313D-4FF3-8D4A-C66D4400DAC9}" name="PivotTable1" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="J17:AM28" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" numFmtId="14" showAll="0">
-      <items count="9">
+      <items count="31">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -2501,38 +2788,61 @@
         <item x="5"/>
         <item x="6"/>
         <item x="7"/>
+        <item x="8"/>
+        <item m="1" x="9"/>
+        <item m="1" x="10"/>
+        <item m="1" x="11"/>
+        <item m="1" x="12"/>
+        <item m="1" x="13"/>
+        <item m="1" x="14"/>
+        <item m="1" x="15"/>
+        <item m="1" x="16"/>
+        <item m="1" x="17"/>
+        <item m="1" x="18"/>
+        <item m="1" x="19"/>
+        <item m="1" x="20"/>
+        <item m="1" x="21"/>
+        <item m="1" x="22"/>
+        <item m="1" x="23"/>
+        <item m="1" x="24"/>
+        <item m="1" x="25"/>
+        <item m="1" x="26"/>
+        <item m="1" x="27"/>
+        <item m="1" x="28"/>
+        <item m="1" x="29"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField axis="axisCol" showAll="0">
-      <items count="28">
-        <item h="1" x="4"/>
-        <item h="1" x="11"/>
-        <item h="1" x="15"/>
-        <item h="1" x="14"/>
-        <item h="1" x="1"/>
-        <item h="1" x="10"/>
-        <item h="1" x="3"/>
-        <item h="1" x="0"/>
-        <item h="1" x="12"/>
-        <item h="1" x="7"/>
-        <item h="1" x="18"/>
-        <item h="1" x="2"/>
-        <item h="1" x="20"/>
-        <item h="1" x="24"/>
-        <item h="1" x="26"/>
-        <item h="1" x="16"/>
-        <item h="1" x="5"/>
-        <item h="1" x="8"/>
-        <item h="1" x="13"/>
-        <item h="1" x="17"/>
-        <item h="1" x="23"/>
-        <item h="1" x="25"/>
-        <item h="1" x="6"/>
+      <items count="29">
+        <item x="4"/>
+        <item x="11"/>
+        <item x="15"/>
+        <item x="14"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="12"/>
+        <item x="7"/>
+        <item x="18"/>
+        <item x="2"/>
+        <item x="20"/>
+        <item x="24"/>
+        <item x="26"/>
+        <item x="16"/>
+        <item x="5"/>
+        <item x="8"/>
+        <item x="13"/>
+        <item x="17"/>
+        <item x="23"/>
+        <item x="25"/>
+        <item x="6"/>
         <item x="19"/>
-        <item h="1" x="21"/>
-        <item h="1" x="22"/>
-        <item h="1" x="9"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="9"/>
+        <item x="27"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -2938,7 +3248,13 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="7">
+  <rowItems count="10">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
     <i>
       <x v="2"/>
     </i>
@@ -2957,6 +3273,9 @@
     <i>
       <x v="7"/>
     </i>
+    <i>
+      <x v="8"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
@@ -2964,9 +3283,90 @@
   <colFields count="1">
     <field x="1"/>
   </colFields>
-  <colItems count="2">
+  <colItems count="29">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
     <i>
       <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
     </i>
     <i t="grand">
       <x/>
@@ -2988,8 +3388,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:H124" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:H124" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:H146" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:H146" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
@@ -3229,7 +3629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:AM146"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -3237,35 +3637,35 @@
     <col min="7" max="8" width="17.75" customWidth="1"/>
     <col min="10" max="10" width="15.75" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.375" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="9.375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.25" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13.125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="15.75" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18.25" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.75" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="11.875" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="18.25" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="15.75" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="18.25" bestFit="1" customWidth="1"/>
@@ -3293,7 +3693,7 @@
     <col min="66" max="66" width="23.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -3319,7 +3719,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>46092</v>
       </c>
@@ -3343,9 +3743,11 @@
         <v>10000000</v>
       </c>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J2" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>46093</v>
       </c>
@@ -3373,13 +3775,13 @@
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="K3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>46093</v>
       </c>
@@ -3406,17 +3808,14 @@
         <v>-666524.9412</v>
       </c>
       <c r="I4" s="2"/>
-      <c r="J4" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J4" s="7">
+        <v>46092</v>
+      </c>
+      <c r="K4" s="2">
+        <v>10000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>46093</v>
       </c>
@@ -3444,16 +3843,13 @@
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="7">
-        <v>46101</v>
-      </c>
-      <c r="K5" s="8">
-        <v>9246</v>
-      </c>
-      <c r="L5" s="8">
-        <v>9246</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46093</v>
+      </c>
+      <c r="K5" s="2">
+        <v>-10000000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>46093</v>
       </c>
@@ -3481,16 +3877,13 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="7">
-        <v>46108</v>
-      </c>
-      <c r="K6" s="8">
-        <v>-1553</v>
-      </c>
-      <c r="L6" s="8">
-        <v>-1553</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46101</v>
+      </c>
+      <c r="K6" s="2">
+        <v>-2665.1533826459199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>46093</v>
       </c>
@@ -3518,16 +3911,13 @@
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="7">
-        <v>46115</v>
-      </c>
-      <c r="K7" s="8">
-        <v>-3861</v>
-      </c>
-      <c r="L7" s="8">
-        <v>-3861</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46108</v>
+      </c>
+      <c r="K7" s="2">
+        <v>-1349.7501089909492</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>46093</v>
       </c>
@@ -3555,16 +3945,13 @@
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="7">
-        <v>46122</v>
-      </c>
-      <c r="K8" s="8">
-        <v>-3049</v>
-      </c>
-      <c r="L8" s="8">
-        <v>-3049</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46115</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1664.5247063139104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>46093</v>
       </c>
@@ -3592,16 +3979,13 @@
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="7">
-        <v>46129</v>
-      </c>
-      <c r="K9" s="8">
-        <v>-1765</v>
-      </c>
-      <c r="L9" s="8">
-        <v>-1765</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46122</v>
+      </c>
+      <c r="K9" s="2">
+        <v>-883.41248167221784</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>46093</v>
       </c>
@@ -3629,16 +4013,13 @@
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="7">
-        <v>46136</v>
-      </c>
-      <c r="K10" s="8">
-        <v>-1055</v>
-      </c>
-      <c r="L10" s="8">
-        <v>-1055</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+        <v>46129</v>
+      </c>
+      <c r="K10" s="2">
+        <v>-73.302777768170927</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>46093</v>
       </c>
@@ -3665,17 +4046,14 @@
         <v>-666627.22489999991</v>
       </c>
       <c r="I11" s="2"/>
-      <c r="J11" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="K11" s="8">
-        <v>-2037</v>
-      </c>
-      <c r="L11" s="8">
-        <v>-2037</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J11" s="7">
+        <v>46136</v>
+      </c>
+      <c r="K11" s="2">
+        <v>736.99024882540107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>46093</v>
       </c>
@@ -3702,8 +4080,14 @@
         <v>-666658.08200000005</v>
       </c>
       <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J12" s="7">
+        <v>46143</v>
+      </c>
+      <c r="K12" s="2">
+        <v>-462.61293519800529</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>46093</v>
       </c>
@@ -3730,8 +4114,14 @@
         <v>-666625.7598</v>
       </c>
       <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K13" s="2">
+        <v>-3032.7167311359517</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>46093</v>
       </c>
@@ -3759,7 +4149,7 @@
       </c>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>46093</v>
       </c>
@@ -3787,7 +4177,7 @@
       </c>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>46093</v>
       </c>
@@ -3814,8 +4204,11 @@
         <v>-666561.89599999995</v>
       </c>
       <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J16" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>46093</v>
       </c>
@@ -3843,13 +4236,13 @@
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="K17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>46093</v>
       </c>
@@ -3876,14 +4269,98 @@
         <v>-1845.7024999987334</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="7">
-        <v>46092</v>
-      </c>
-      <c r="K18" s="2">
-        <v>10000000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J18" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K18" t="s">
+        <v>8</v>
+      </c>
+      <c r="L18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M18" t="s">
+        <v>19</v>
+      </c>
+      <c r="N18" t="s">
+        <v>18</v>
+      </c>
+      <c r="O18" t="s">
+        <v>5</v>
+      </c>
+      <c r="P18" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>7</v>
+      </c>
+      <c r="R18" t="s">
+        <v>29</v>
+      </c>
+      <c r="S18" t="s">
+        <v>16</v>
+      </c>
+      <c r="T18" t="s">
+        <v>11</v>
+      </c>
+      <c r="U18" t="s">
+        <v>25</v>
+      </c>
+      <c r="V18" t="s">
+        <v>6</v>
+      </c>
+      <c r="W18" t="s">
+        <v>32</v>
+      </c>
+      <c r="X18" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>20</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>9</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>37</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI18" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ18" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK18" t="s">
+        <v>13</v>
+      </c>
+      <c r="AL18" t="s">
+        <v>45</v>
+      </c>
+      <c r="AM18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>46101</v>
       </c>
@@ -3910,13 +4387,43 @@
         <v>-14418.705749999999</v>
       </c>
       <c r="J19" s="7">
-        <v>46093</v>
-      </c>
-      <c r="K19" s="2">
+        <v>46092</v>
+      </c>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10">
         <v>-10000000</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="10"/>
+      <c r="Y19" s="10"/>
+      <c r="Z19" s="10"/>
+      <c r="AA19" s="10"/>
+      <c r="AB19" s="10"/>
+      <c r="AC19" s="10"/>
+      <c r="AD19" s="10"/>
+      <c r="AE19" s="10"/>
+      <c r="AF19" s="10"/>
+      <c r="AG19" s="10"/>
+      <c r="AH19" s="10"/>
+      <c r="AI19" s="10"/>
+      <c r="AJ19" s="10"/>
+      <c r="AK19" s="10"/>
+      <c r="AL19" s="10"/>
+      <c r="AM19" s="10">
+        <v>-10000000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>46101</v>
       </c>
@@ -3943,13 +4450,73 @@
         <v>-2591.7952500000001</v>
       </c>
       <c r="J20" s="7">
-        <v>46101</v>
-      </c>
-      <c r="K20" s="2">
-        <v>-2665.1533826459199</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46093</v>
+      </c>
+      <c r="K20" s="10">
+        <v>4716</v>
+      </c>
+      <c r="L20" s="10">
+        <v>726</v>
+      </c>
+      <c r="M20" s="10">
+        <v>3871</v>
+      </c>
+      <c r="N20" s="10">
+        <v>1081</v>
+      </c>
+      <c r="O20" s="10">
+        <v>564</v>
+      </c>
+      <c r="P20" s="10">
+        <v>17020</v>
+      </c>
+      <c r="Q20" s="10">
+        <v>36623</v>
+      </c>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10">
+        <v>25909</v>
+      </c>
+      <c r="T20" s="10">
+        <v>3159</v>
+      </c>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10">
+        <v>4362</v>
+      </c>
+      <c r="W20" s="10"/>
+      <c r="X20" s="10"/>
+      <c r="Y20" s="10"/>
+      <c r="Z20" s="10">
+        <v>366.96075312617717</v>
+      </c>
+      <c r="AA20" s="10">
+        <v>14659</v>
+      </c>
+      <c r="AB20" s="10">
+        <v>2276</v>
+      </c>
+      <c r="AC20" s="10">
+        <v>429</v>
+      </c>
+      <c r="AD20" s="10"/>
+      <c r="AE20" s="10"/>
+      <c r="AF20" s="10"/>
+      <c r="AG20" s="10">
+        <v>3987</v>
+      </c>
+      <c r="AH20" s="10"/>
+      <c r="AI20" s="10"/>
+      <c r="AJ20" s="10"/>
+      <c r="AK20" s="10">
+        <v>9919</v>
+      </c>
+      <c r="AL20" s="10"/>
+      <c r="AM20" s="10">
+        <v>129667.96075312617</v>
+      </c>
+    </row>
+    <row r="21" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>46101</v>
       </c>
@@ -3976,13 +4543,77 @@
         <v>-43123.091263257927</v>
       </c>
       <c r="J21" s="7">
-        <v>46108</v>
-      </c>
-      <c r="K21" s="2">
-        <v>-1349.7501089909492</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46101</v>
+      </c>
+      <c r="K21" s="10">
+        <v>1</v>
+      </c>
+      <c r="L21" s="10">
+        <v>3</v>
+      </c>
+      <c r="M21" s="10">
+        <v>-3871</v>
+      </c>
+      <c r="N21" s="10">
+        <v>-4</v>
+      </c>
+      <c r="O21" s="10">
+        <v>-5</v>
+      </c>
+      <c r="P21" s="10">
+        <v>-612</v>
+      </c>
+      <c r="Q21" s="10">
+        <v>-36623</v>
+      </c>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10">
+        <v>-472</v>
+      </c>
+      <c r="T21" s="10">
+        <v>74</v>
+      </c>
+      <c r="U21" s="10">
+        <v>26650</v>
+      </c>
+      <c r="V21" s="10">
+        <v>112</v>
+      </c>
+      <c r="W21" s="10"/>
+      <c r="X21" s="10"/>
+      <c r="Y21" s="10"/>
+      <c r="Z21" s="10"/>
+      <c r="AA21" s="10">
+        <v>1077</v>
+      </c>
+      <c r="AB21" s="10">
+        <v>24</v>
+      </c>
+      <c r="AC21" s="10">
+        <v>-429</v>
+      </c>
+      <c r="AD21" s="10">
+        <v>380</v>
+      </c>
+      <c r="AE21" s="10"/>
+      <c r="AF21" s="10"/>
+      <c r="AG21" s="10">
+        <v>107</v>
+      </c>
+      <c r="AH21" s="10">
+        <v>9246</v>
+      </c>
+      <c r="AI21" s="10"/>
+      <c r="AJ21" s="10"/>
+      <c r="AK21" s="10">
+        <v>-294</v>
+      </c>
+      <c r="AL21" s="10"/>
+      <c r="AM21" s="10">
+        <v>-4636</v>
+      </c>
+    </row>
+    <row r="22" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>46101</v>
       </c>
@@ -4009,13 +4640,85 @@
         <v>-15771.881999999887</v>
       </c>
       <c r="J22" s="7">
-        <v>46115</v>
-      </c>
-      <c r="K22" s="2">
-        <v>1664.5247063139104</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46108</v>
+      </c>
+      <c r="K22" s="10">
+        <v>-2845</v>
+      </c>
+      <c r="L22" s="10">
+        <v>-431</v>
+      </c>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10">
+        <v>-1077</v>
+      </c>
+      <c r="O22" s="10">
+        <v>279</v>
+      </c>
+      <c r="P22" s="10">
+        <v>-1609</v>
+      </c>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+      <c r="S22" s="10">
+        <v>-13938</v>
+      </c>
+      <c r="T22" s="10">
+        <v>-3233</v>
+      </c>
+      <c r="U22" s="10">
+        <v>34714</v>
+      </c>
+      <c r="V22" s="10">
+        <v>-321</v>
+      </c>
+      <c r="W22" s="10">
+        <v>5846</v>
+      </c>
+      <c r="X22" s="10">
+        <v>34709</v>
+      </c>
+      <c r="Y22" s="10"/>
+      <c r="Z22" s="10"/>
+      <c r="AA22" s="10">
+        <v>-15736</v>
+      </c>
+      <c r="AB22" s="10">
+        <v>-2300</v>
+      </c>
+      <c r="AC22" s="10">
+        <v>221</v>
+      </c>
+      <c r="AD22" s="10">
+        <v>-380</v>
+      </c>
+      <c r="AE22" s="10">
+        <v>1724</v>
+      </c>
+      <c r="AF22" s="10">
+        <v>56041</v>
+      </c>
+      <c r="AG22" s="10">
+        <v>-4094</v>
+      </c>
+      <c r="AH22" s="10">
+        <v>-1553</v>
+      </c>
+      <c r="AI22" s="10">
+        <v>18700</v>
+      </c>
+      <c r="AJ22" s="10">
+        <v>12173</v>
+      </c>
+      <c r="AK22" s="10">
+        <v>-9625</v>
+      </c>
+      <c r="AL22" s="10"/>
+      <c r="AM22" s="10">
+        <v>107265</v>
+      </c>
+    </row>
+    <row r="23" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>46101</v>
       </c>
@@ -4042,13 +4745,73 @@
         <v>-133.56674999999899</v>
       </c>
       <c r="J23" s="7">
-        <v>46122</v>
-      </c>
-      <c r="K23" s="2">
-        <v>-883.41248167221784</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46115</v>
+      </c>
+      <c r="K23" s="10">
+        <v>947</v>
+      </c>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10">
+        <v>314</v>
+      </c>
+      <c r="P23" s="10">
+        <v>7328</v>
+      </c>
+      <c r="Q23" s="10">
+        <v>37957</v>
+      </c>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10">
+        <v>1216</v>
+      </c>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10">
+        <v>-12852</v>
+      </c>
+      <c r="V23" s="10">
+        <v>-2461</v>
+      </c>
+      <c r="W23" s="10">
+        <v>6143</v>
+      </c>
+      <c r="X23" s="10">
+        <v>-5905</v>
+      </c>
+      <c r="Y23" s="10"/>
+      <c r="Z23" s="10"/>
+      <c r="AA23" s="10"/>
+      <c r="AB23" s="10">
+        <v>782</v>
+      </c>
+      <c r="AC23" s="10">
+        <v>-221</v>
+      </c>
+      <c r="AD23" s="10"/>
+      <c r="AE23" s="10">
+        <v>246</v>
+      </c>
+      <c r="AF23" s="10">
+        <v>-4227</v>
+      </c>
+      <c r="AG23" s="10"/>
+      <c r="AH23" s="10">
+        <v>-3861</v>
+      </c>
+      <c r="AI23" s="10">
+        <v>2177</v>
+      </c>
+      <c r="AJ23" s="10">
+        <v>-12173</v>
+      </c>
+      <c r="AK23" s="10"/>
+      <c r="AL23" s="10"/>
+      <c r="AM23" s="10">
+        <v>15410</v>
+      </c>
+    </row>
+    <row r="24" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>46101</v>
       </c>
@@ -4075,13 +4838,71 @@
         <v>-6574.4853068847597</v>
       </c>
       <c r="J24" s="7">
-        <v>46129</v>
-      </c>
-      <c r="K24" s="2">
-        <v>-73.302777768170927</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46122</v>
+      </c>
+      <c r="K24" s="10">
+        <v>1900</v>
+      </c>
+      <c r="L24" s="10">
+        <v>-294</v>
+      </c>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10">
+        <v>-569</v>
+      </c>
+      <c r="P24" s="10">
+        <v>5804</v>
+      </c>
+      <c r="Q24" s="10">
+        <v>-36557</v>
+      </c>
+      <c r="R24" s="10"/>
+      <c r="S24" s="10">
+        <v>663</v>
+      </c>
+      <c r="T24" s="10"/>
+      <c r="U24" s="10">
+        <v>-3328</v>
+      </c>
+      <c r="V24" s="10">
+        <v>6951</v>
+      </c>
+      <c r="W24" s="10">
+        <v>-2481</v>
+      </c>
+      <c r="X24" s="10"/>
+      <c r="Y24" s="10"/>
+      <c r="Z24" s="10"/>
+      <c r="AA24" s="10">
+        <v>2584</v>
+      </c>
+      <c r="AB24" s="10">
+        <v>-115</v>
+      </c>
+      <c r="AC24" s="10"/>
+      <c r="AD24" s="10"/>
+      <c r="AE24" s="10">
+        <v>-400</v>
+      </c>
+      <c r="AF24" s="10">
+        <v>19597</v>
+      </c>
+      <c r="AG24" s="10"/>
+      <c r="AH24" s="10">
+        <v>-3049</v>
+      </c>
+      <c r="AI24" s="10">
+        <v>3599</v>
+      </c>
+      <c r="AJ24" s="10"/>
+      <c r="AK24" s="10"/>
+      <c r="AL24" s="10"/>
+      <c r="AM24" s="10">
+        <v>-5695</v>
+      </c>
+    </row>
+    <row r="25" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>46101</v>
       </c>
@@ -4108,13 +4929,77 @@
         <v>-16466.970154083159</v>
       </c>
       <c r="J25" s="7">
-        <v>46136</v>
-      </c>
-      <c r="K25" s="2">
-        <v>736.99024882540107</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>46129</v>
+      </c>
+      <c r="K25" s="10">
+        <v>-1401</v>
+      </c>
+      <c r="L25" s="10">
+        <v>-81</v>
+      </c>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10">
+        <v>674</v>
+      </c>
+      <c r="P25" s="10">
+        <v>19134</v>
+      </c>
+      <c r="Q25" s="10">
+        <v>832</v>
+      </c>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10">
+        <v>6891</v>
+      </c>
+      <c r="T25" s="10"/>
+      <c r="U25" s="10">
+        <v>-938</v>
+      </c>
+      <c r="V25" s="10">
+        <v>-4228</v>
+      </c>
+      <c r="W25" s="10">
+        <v>-6028</v>
+      </c>
+      <c r="X25" s="10"/>
+      <c r="Y25" s="10">
+        <v>4327</v>
+      </c>
+      <c r="Z25" s="10"/>
+      <c r="AA25" s="10">
+        <v>-803</v>
+      </c>
+      <c r="AB25" s="10">
+        <v>-1010</v>
+      </c>
+      <c r="AC25" s="10"/>
+      <c r="AD25" s="10"/>
+      <c r="AE25" s="10">
+        <v>-1147</v>
+      </c>
+      <c r="AF25" s="10">
+        <v>-50484</v>
+      </c>
+      <c r="AG25" s="10">
+        <v>1388</v>
+      </c>
+      <c r="AH25" s="10">
+        <v>-1765</v>
+      </c>
+      <c r="AI25" s="10">
+        <v>2329</v>
+      </c>
+      <c r="AJ25" s="10"/>
+      <c r="AK25" s="10">
+        <v>3946</v>
+      </c>
+      <c r="AL25" s="10"/>
+      <c r="AM25" s="10">
+        <v>-28364</v>
+      </c>
+    </row>
+    <row r="26" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>46101</v>
       </c>
@@ -4140,14 +5025,76 @@
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>-629594.64</v>
       </c>
-      <c r="J26" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="K26" s="2">
-        <v>-2570.1037959379464</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J26" s="7">
+        <v>46136</v>
+      </c>
+      <c r="K26" s="10">
+        <v>-577</v>
+      </c>
+      <c r="L26" s="10">
+        <v>175</v>
+      </c>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10">
+        <v>-111</v>
+      </c>
+      <c r="P26" s="10">
+        <v>-27490</v>
+      </c>
+      <c r="Q26" s="10">
+        <v>9644</v>
+      </c>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10">
+        <v>-7468</v>
+      </c>
+      <c r="T26" s="10"/>
+      <c r="U26" s="10">
+        <v>10225</v>
+      </c>
+      <c r="V26" s="10">
+        <v>3623</v>
+      </c>
+      <c r="W26" s="10">
+        <v>11124</v>
+      </c>
+      <c r="X26" s="10"/>
+      <c r="Y26" s="10">
+        <v>23473</v>
+      </c>
+      <c r="Z26" s="10"/>
+      <c r="AA26" s="10">
+        <v>2251</v>
+      </c>
+      <c r="AB26" s="10"/>
+      <c r="AC26" s="10">
+        <v>225</v>
+      </c>
+      <c r="AD26" s="10"/>
+      <c r="AE26" s="10">
+        <v>-1247</v>
+      </c>
+      <c r="AF26" s="10"/>
+      <c r="AG26" s="10">
+        <v>208</v>
+      </c>
+      <c r="AH26" s="10">
+        <v>-1055</v>
+      </c>
+      <c r="AI26" s="10">
+        <v>-22074</v>
+      </c>
+      <c r="AJ26" s="10"/>
+      <c r="AK26" s="10">
+        <v>1059</v>
+      </c>
+      <c r="AL26" s="10"/>
+      <c r="AM26" s="10">
+        <v>1985</v>
+      </c>
+    </row>
+    <row r="27" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>46101</v>
       </c>
@@ -4173,8 +5120,86 @@
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>-629787.75887675246</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J27" s="7">
+        <v>46143</v>
+      </c>
+      <c r="K27" s="10">
+        <v>-2741</v>
+      </c>
+      <c r="L27" s="10">
+        <v>147</v>
+      </c>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10">
+        <v>101</v>
+      </c>
+      <c r="P27" s="10">
+        <v>15813</v>
+      </c>
+      <c r="Q27" s="10">
+        <v>26551</v>
+      </c>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10">
+        <v>11411</v>
+      </c>
+      <c r="T27" s="10"/>
+      <c r="U27" s="10">
+        <v>9077</v>
+      </c>
+      <c r="V27" s="10">
+        <v>380</v>
+      </c>
+      <c r="W27" s="10">
+        <v>-3779</v>
+      </c>
+      <c r="X27" s="10">
+        <v>-28804</v>
+      </c>
+      <c r="Y27" s="10">
+        <v>-27800</v>
+      </c>
+      <c r="Z27" s="10"/>
+      <c r="AA27" s="10">
+        <v>1204</v>
+      </c>
+      <c r="AB27" s="10">
+        <v>343</v>
+      </c>
+      <c r="AC27" s="10">
+        <v>-7</v>
+      </c>
+      <c r="AD27" s="10">
+        <v>130</v>
+      </c>
+      <c r="AE27" s="10">
+        <v>824</v>
+      </c>
+      <c r="AF27" s="10">
+        <v>14533</v>
+      </c>
+      <c r="AG27" s="10">
+        <v>-96</v>
+      </c>
+      <c r="AH27" s="10">
+        <v>2037</v>
+      </c>
+      <c r="AI27" s="10">
+        <v>-4731</v>
+      </c>
+      <c r="AJ27" s="10"/>
+      <c r="AK27" s="10">
+        <v>-1215</v>
+      </c>
+      <c r="AL27" s="10">
+        <v>4104</v>
+      </c>
+      <c r="AM27" s="10">
+        <v>17482</v>
+      </c>
+    </row>
+    <row r="28" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>46101</v>
       </c>
@@ -4200,8 +5225,98 @@
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>-629782.43077839643</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J28" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K28" s="10">
+        <v>0</v>
+      </c>
+      <c r="L28" s="10">
+        <v>245</v>
+      </c>
+      <c r="M28" s="10">
+        <v>0</v>
+      </c>
+      <c r="N28" s="10">
+        <v>0</v>
+      </c>
+      <c r="O28" s="10">
+        <v>1247</v>
+      </c>
+      <c r="P28" s="10">
+        <v>35388</v>
+      </c>
+      <c r="Q28" s="10">
+        <v>38427</v>
+      </c>
+      <c r="R28" s="10">
+        <v>-10000000</v>
+      </c>
+      <c r="S28" s="10">
+        <v>24212</v>
+      </c>
+      <c r="T28" s="10">
+        <v>0</v>
+      </c>
+      <c r="U28" s="10">
+        <v>63548</v>
+      </c>
+      <c r="V28" s="10">
+        <v>8418</v>
+      </c>
+      <c r="W28" s="10">
+        <v>10825</v>
+      </c>
+      <c r="X28" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="10">
+        <v>366.96075312617717</v>
+      </c>
+      <c r="AA28" s="10">
+        <v>5236</v>
+      </c>
+      <c r="AB28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="10">
+        <v>218</v>
+      </c>
+      <c r="AD28" s="10">
+        <v>130</v>
+      </c>
+      <c r="AE28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="10">
+        <v>35460</v>
+      </c>
+      <c r="AG28" s="10">
+        <v>1500</v>
+      </c>
+      <c r="AH28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AI28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AK28" s="10">
+        <v>3790</v>
+      </c>
+      <c r="AL28" s="10">
+        <v>4104</v>
+      </c>
+      <c r="AM28" s="10">
+        <v>-9766885.0392468739</v>
+      </c>
+    </row>
+    <row r="29" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>46101</v>
       </c>
@@ -4228,7 +5343,7 @@
         <v>19229.741037414537</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>46101</v>
       </c>
@@ -4255,7 +5370,7 @@
         <v>2338.0303511962879</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>46101</v>
       </c>
@@ -4282,7 +5397,7 @@
         <v>23479.873163291908</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>46101</v>
       </c>
@@ -5460,7 +6575,7 @@
         <v>41.555000305175703</v>
       </c>
       <c r="F75">
-        <v>2.0777500152587801E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G75" s="2">
         <v>41.5757778053283</v>
@@ -5487,7 +6602,7 @@
         <v>10.5159997940063</v>
       </c>
       <c r="F76">
-        <v>5.2579998970031698E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G76" s="2">
         <v>10.521257793903301</v>
@@ -5514,7 +6629,7 @@
         <v>167.22000122070301</v>
       </c>
       <c r="F77">
-        <v>8.3610000610351495E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G77" s="2">
         <v>167.30361122131299</v>
@@ -5541,7 +6656,7 @@
         <v>27.709999084472599</v>
       </c>
       <c r="F78">
-        <v>1.3854999542236301E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G78" s="2">
         <v>27.7238540840148</v>
@@ -5568,7 +6683,7 @@
         <v>137.80000305175699</v>
       </c>
       <c r="F79">
-        <v>6.8900001525878898E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G79" s="2">
         <v>137.86890305328299</v>
@@ -5595,7 +6710,7 @@
         <v>78.610000610351506</v>
       </c>
       <c r="F80">
-        <v>3.9305000305175697E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G80" s="2">
         <v>78.649305610656697</v>
@@ -5622,7 +6737,7 @@
         <v>40.119998931884702</v>
       </c>
       <c r="F81">
-        <v>2.0059999465942301E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G81" s="2">
         <v>40.140058931350701</v>
@@ -5649,7 +6764,7 @@
         <v>23.9500007629394</v>
       </c>
       <c r="F82">
-        <v>1.1975000381469701E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G82" s="2">
         <v>23.938025762557899</v>
@@ -5676,7 +6791,7 @@
         <v>19.704999923706001</v>
       </c>
       <c r="F83">
-        <v>9.8524999618530198E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G83" s="2">
         <v>19.695147423744199</v>
@@ -5703,7 +6818,7 @@
         <v>313.29998779296801</v>
       </c>
       <c r="F84">
-        <v>0.15664999389648401</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G84" s="2">
         <v>313.14333779907201</v>
@@ -5730,7 +6845,7 @@
         <v>858.79998779296795</v>
       </c>
       <c r="F85">
-        <v>0.42939999389648398</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G85" s="2">
         <v>858.37058779907204</v>
@@ -5757,7 +6872,7 @@
         <v>76</v>
       </c>
       <c r="F86">
-        <v>3.7999999999999999E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G86" s="2">
         <v>75.962000000000003</v>
@@ -5784,7 +6899,7 @@
         <v>1270</v>
       </c>
       <c r="F87">
-        <v>0.63500000000000001</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G87" s="2">
         <v>1269.365</v>
@@ -5811,7 +6926,7 @@
         <v>42.825000762939403</v>
       </c>
       <c r="F88">
-        <v>2.1412500381469701E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G88" s="2">
         <v>42.803588262557902</v>
@@ -5838,7 +6953,7 @@
         <v>301.64999389648398</v>
       </c>
       <c r="F89">
-        <v>0.150824996948242</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G89" s="2">
         <v>301.49916889953602</v>
@@ -6351,7 +7466,7 @@
         <v>41.534999847412102</v>
       </c>
       <c r="F108">
-        <v>2.0767499923705999E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G108" s="2">
         <v>41.555767347335802</v>
@@ -6378,7 +7493,7 @@
         <v>22.9500007629394</v>
       </c>
       <c r="F109">
-        <v>1.14750003814697E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G109" s="2">
         <v>22.961475763320902</v>
@@ -6405,7 +7520,7 @@
         <v>18.579999923706001</v>
       </c>
       <c r="F110">
-        <v>9.2899999618530193E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G110" s="2">
         <v>18.589289923667899</v>
@@ -6432,7 +7547,7 @@
         <v>147.27999877929599</v>
       </c>
       <c r="F111">
-        <v>7.3639999389648395E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G111" s="2">
         <v>147.35363877868599</v>
@@ -6459,7 +7574,7 @@
         <v>52.560001373291001</v>
       </c>
       <c r="F112">
-        <v>2.6280000686645499E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G112" s="2">
         <v>52.586281373977599</v>
@@ -6486,7 +7601,7 @@
         <v>66.419998168945298</v>
       </c>
       <c r="F113">
-        <v>3.32099990844726E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G113" s="2">
         <v>66.453208168029704</v>
@@ -6513,7 +7628,7 @@
         <v>975.09997558593705</v>
       </c>
       <c r="F114">
-        <v>0.48754998779296799</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G114" s="2">
         <v>975.58752557372998</v>
@@ -6540,7 +7655,7 @@
         <v>1319.19995117187</v>
       </c>
       <c r="F115">
-        <v>0.65959997558593697</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G115" s="2">
         <v>1319.85955114746</v>
@@ -6567,7 +7682,7 @@
         <v>54.150001525878899</v>
       </c>
       <c r="F116">
-        <v>2.7075000762939401E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G116" s="2">
         <v>54.177076526641798</v>
@@ -6594,7 +7709,7 @@
         <v>187.61999511718699</v>
       </c>
       <c r="F117">
-        <v>9.3809997558593705E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G117" s="2">
         <v>187.71380511474601</v>
@@ -6621,7 +7736,7 @@
         <v>77.540000915527301</v>
       </c>
       <c r="F118">
-        <v>3.8770000457763597E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G118" s="2">
         <v>77.501230915069499</v>
@@ -6648,7 +7763,7 @@
         <v>1249.59997558593</v>
       </c>
       <c r="F119">
-        <v>0.62479998779296797</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G119" s="2">
         <v>1248.9751755981399</v>
@@ -6675,7 +7790,7 @@
         <v>136.25</v>
       </c>
       <c r="F120">
-        <v>6.8125000000000005E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G120" s="2">
         <v>136.18187499999999</v>
@@ -6702,7 +7817,7 @@
         <v>38.5</v>
       </c>
       <c r="F121">
-        <v>1.925E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G121" s="2">
         <v>38.48075</v>
@@ -6729,7 +7844,7 @@
         <v>27.059999465942301</v>
       </c>
       <c r="F122">
-        <v>1.35299997329711E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G122" s="2">
         <v>27.046469466209398</v>
@@ -6756,7 +7871,7 @@
         <v>270</v>
       </c>
       <c r="F123">
-        <v>0.13500000000000001</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G123" s="2">
         <v>269.86500000000001</v>
@@ -6783,7 +7898,7 @@
         <v>77</v>
       </c>
       <c r="F124">
-        <v>3.85E-2</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="G124" s="2">
         <v>76.961500000000001</v>
@@ -6791,6 +7906,600 @@
       <c r="H124" s="2">
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>1698848.1510000001</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B125" t="s">
+        <v>28</v>
+      </c>
+      <c r="C125" t="s">
+        <v>23</v>
+      </c>
+      <c r="D125">
+        <v>2037</v>
+      </c>
+      <c r="E125" s="2">
+        <v>77.639999000000003</v>
+      </c>
+      <c r="F125">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G125" s="2">
+        <v>77.678818999499995</v>
+      </c>
+      <c r="H125" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-158231.75430198148</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B126" t="s">
+        <v>12</v>
+      </c>
+      <c r="C126" t="s">
+        <v>23</v>
+      </c>
+      <c r="D126">
+        <v>343</v>
+      </c>
+      <c r="E126" s="2">
+        <v>293.35000600000001</v>
+      </c>
+      <c r="F126">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G126" s="2">
+        <v>293.49668100299999</v>
+      </c>
+      <c r="H126" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-100669.361584029</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B127" t="s">
+        <v>35</v>
+      </c>
+      <c r="C127" t="s">
+        <v>23</v>
+      </c>
+      <c r="D127">
+        <v>824</v>
+      </c>
+      <c r="E127" s="2">
+        <v>273</v>
+      </c>
+      <c r="F127">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G127" s="2">
+        <v>273.13650000000001</v>
+      </c>
+      <c r="H127" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-225064.47600000002</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B128" t="s">
+        <v>16</v>
+      </c>
+      <c r="C128" t="s">
+        <v>23</v>
+      </c>
+      <c r="D128">
+        <v>11411</v>
+      </c>
+      <c r="E128" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="F128">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G128" s="2">
+        <v>26.513249999999999</v>
+      </c>
+      <c r="H128" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-302542.69575000001</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B129" t="s">
+        <v>37</v>
+      </c>
+      <c r="C129" t="s">
+        <v>23</v>
+      </c>
+      <c r="D129">
+        <v>14533</v>
+      </c>
+      <c r="E129" s="2">
+        <v>10.3800001144409</v>
+      </c>
+      <c r="F129">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G129" s="2">
+        <v>10.3851901144981</v>
+      </c>
+      <c r="H129" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-150927.96793400089</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B130" t="s">
+        <v>27</v>
+      </c>
+      <c r="C130" t="s">
+        <v>23</v>
+      </c>
+      <c r="D130">
+        <v>130</v>
+      </c>
+      <c r="E130" s="2">
+        <v>1623.5</v>
+      </c>
+      <c r="F130">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G130" s="2">
+        <v>1624.3117499999901</v>
+      </c>
+      <c r="H130" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-211160.52749999872</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B131" t="s">
+        <v>45</v>
+      </c>
+      <c r="C131" t="s">
+        <v>23</v>
+      </c>
+      <c r="D131">
+        <v>4104</v>
+      </c>
+      <c r="E131" s="2">
+        <v>89.230003356933594</v>
+      </c>
+      <c r="F131">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G131" s="2">
+        <v>89.274618358612003</v>
+      </c>
+      <c r="H131" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-366383.03374374367</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B132" t="s">
+        <v>6</v>
+      </c>
+      <c r="C132" t="s">
+        <v>23</v>
+      </c>
+      <c r="D132">
+        <v>380</v>
+      </c>
+      <c r="E132" s="2">
+        <v>180.58000183105401</v>
+      </c>
+      <c r="F132">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G132" s="2">
+        <v>180.67029183196999</v>
+      </c>
+      <c r="H132" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-68654.710896148594</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B133" t="s">
+        <v>9</v>
+      </c>
+      <c r="C133" t="s">
+        <v>23</v>
+      </c>
+      <c r="D133">
+        <v>1204</v>
+      </c>
+      <c r="E133" s="2">
+        <v>41.069999694824197</v>
+      </c>
+      <c r="F133">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G133" s="2">
+        <v>41.090534694671597</v>
+      </c>
+      <c r="H133" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-49473.003772384604</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B134" t="s">
+        <v>25</v>
+      </c>
+      <c r="C134" t="s">
+        <v>23</v>
+      </c>
+      <c r="D134">
+        <v>9077</v>
+      </c>
+      <c r="E134" s="2">
+        <v>24</v>
+      </c>
+      <c r="F134">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G134" s="2">
+        <v>24.012</v>
+      </c>
+      <c r="H134" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-217956.924</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B135" t="s">
+        <v>14</v>
+      </c>
+      <c r="C135" t="s">
+        <v>23</v>
+      </c>
+      <c r="D135">
+        <v>15813</v>
+      </c>
+      <c r="E135" s="2">
+        <v>38.049999237060497</v>
+      </c>
+      <c r="F135">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G135" s="2">
+        <v>38.069024236678999</v>
+      </c>
+      <c r="H135" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-601985.48025460506</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B136" t="s">
+        <v>15</v>
+      </c>
+      <c r="C136" t="s">
+        <v>23</v>
+      </c>
+      <c r="D136">
+        <v>147</v>
+      </c>
+      <c r="E136" s="2">
+        <v>958.5</v>
+      </c>
+      <c r="F136">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G136" s="2">
+        <v>958.97924999999998</v>
+      </c>
+      <c r="H136" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-140969.94975</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B137" t="s">
+        <v>5</v>
+      </c>
+      <c r="C137" t="s">
+        <v>23</v>
+      </c>
+      <c r="D137">
+        <v>101</v>
+      </c>
+      <c r="E137" s="2">
+        <v>1222.40002441406</v>
+      </c>
+      <c r="F137">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G137" s="2">
+        <v>1223.01122442626</v>
+      </c>
+      <c r="H137" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-123524.13366705226</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B138" t="s">
+        <v>7</v>
+      </c>
+      <c r="C138" t="s">
+        <v>23</v>
+      </c>
+      <c r="D138">
+        <v>26551</v>
+      </c>
+      <c r="E138" s="2">
+        <v>18.809999465942301</v>
+      </c>
+      <c r="F138">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G138" s="2">
+        <v>18.819404465675301</v>
+      </c>
+      <c r="H138" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-499674.00796814496</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B139" t="s">
+        <v>13</v>
+      </c>
+      <c r="C139" t="s">
+        <v>26</v>
+      </c>
+      <c r="D139">
+        <v>-1215</v>
+      </c>
+      <c r="E139" s="2">
+        <v>66.419998168945298</v>
+      </c>
+      <c r="F139">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G139" s="2">
+        <v>66.386788169860793</v>
+      </c>
+      <c r="H139" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>80659.947626380861</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B140" t="s">
+        <v>10</v>
+      </c>
+      <c r="C140" t="s">
+        <v>26</v>
+      </c>
+      <c r="D140">
+        <v>-96</v>
+      </c>
+      <c r="E140" s="2">
+        <v>145.5</v>
+      </c>
+      <c r="F140">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G140" s="2">
+        <v>145.42724999999999</v>
+      </c>
+      <c r="H140" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>13961.016</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B141" t="s">
+        <v>33</v>
+      </c>
+      <c r="C141" t="s">
+        <v>26</v>
+      </c>
+      <c r="D141">
+        <v>-4731</v>
+      </c>
+      <c r="E141" s="2">
+        <v>79.290000915527301</v>
+      </c>
+      <c r="F141">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G141" s="2">
+        <v>79.250355915069505</v>
+      </c>
+      <c r="H141" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>374933.43383419386</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B142" t="s">
+        <v>36</v>
+      </c>
+      <c r="C142" t="s">
+        <v>26</v>
+      </c>
+      <c r="D142">
+        <v>-28804</v>
+      </c>
+      <c r="E142" s="2">
+        <v>24.754999160766602</v>
+      </c>
+      <c r="F142">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G142" s="2">
+        <v>24.742621661186199</v>
+      </c>
+      <c r="H142" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>712686.47432880732</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B143" t="s">
+        <v>8</v>
+      </c>
+      <c r="C143" t="s">
+        <v>26</v>
+      </c>
+      <c r="D143">
+        <v>-2741</v>
+      </c>
+      <c r="E143" s="2">
+        <v>147.39999389648401</v>
+      </c>
+      <c r="F143">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G143" s="2">
+        <v>147.32629389953601</v>
+      </c>
+      <c r="H143" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>403821.3715786282</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>38</v>
+      </c>
+      <c r="C144" t="s">
+        <v>26</v>
+      </c>
+      <c r="D144">
+        <v>-27800</v>
+      </c>
+      <c r="E144" s="2">
+        <v>50.580001831054602</v>
+      </c>
+      <c r="F144">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G144" s="2">
+        <v>50.554711830139098</v>
+      </c>
+      <c r="H144" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>1405420.9888778669</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B145" t="s">
+        <v>17</v>
+      </c>
+      <c r="C145" t="s">
+        <v>26</v>
+      </c>
+      <c r="D145">
+        <v>-7</v>
+      </c>
+      <c r="E145" s="2">
+        <v>1355.80004882812</v>
+      </c>
+      <c r="F145">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G145" s="2">
+        <v>1355.1221488037099</v>
+      </c>
+      <c r="H145" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>9485.8550416259695</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A146" s="4">
+        <v>46143</v>
+      </c>
+      <c r="B146" t="s">
+        <v>32</v>
+      </c>
+      <c r="C146" t="s">
+        <v>26</v>
+      </c>
+      <c r="D146">
+        <v>-3779</v>
+      </c>
+      <c r="E146" s="2">
+        <v>57.130001068115199</v>
+      </c>
+      <c r="F146">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G146" s="2">
+        <v>57.101436067581098</v>
+      </c>
+      <c r="H146" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>215786.32689938898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Envío 8 de mayo
</commit_message>
<xml_diff>
--- a/Envíos/historico_operativa.xlsx
+++ b/Envíos/historico_operativa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deportivo Estadio\Desktop\Master Quant\Gestión de activos\Trabajo gestión cuantitativa\Trabajo_gestion_cuantitativa\Trabajo_gestion_cuantitativa\Envíos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FB0ABF-1B28-413B-A3EC-18775D89F40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CD1A9E-9424-4FE7-9843-6AF88B21F346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Operativa" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="43" r:id="rId3"/>
+    <pivotCache cacheId="5" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -332,7 +332,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="estadio gijon" refreshedDate="46143.824766203703" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="145" xr:uid="{F974E3A8-FD59-40A3-ACE6-0C536987A82A}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="estadio gijon" refreshedDate="46150.760364120368" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="161" xr:uid="{F974E3A8-FD59-40A3-ACE6-0C536987A82A}">
   <cacheSource type="worksheet">
     <worksheetSource name="Operaciones_table"/>
   </cacheSource>
@@ -348,13 +348,13 @@
         <d v="2026-04-17T00:00:00"/>
         <d v="2026-04-24T00:00:00"/>
         <d v="2026-05-01T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
         <d v="2026-05-02T00:00:00" u="1"/>
         <d v="2026-05-03T00:00:00" u="1"/>
         <d v="2026-05-04T00:00:00" u="1"/>
         <d v="2026-05-05T00:00:00" u="1"/>
         <d v="2026-05-06T00:00:00" u="1"/>
         <d v="2026-05-07T00:00:00" u="1"/>
-        <d v="2026-05-08T00:00:00" u="1"/>
         <d v="2026-05-09T00:00:00" u="1"/>
         <d v="2026-05-10T00:00:00" u="1"/>
         <d v="2026-05-11T00:00:00" u="1"/>
@@ -411,20 +411,20 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-10000000" maxValue="56041"/>
     </cacheField>
     <cacheField name="Precio" numFmtId="6">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1" maxValue="1656"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1" maxValue="1661"/>
     </cacheField>
     <cacheField name="CT" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.0000000000000001E-4" maxValue="5.0000000000000001E-4"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.0000000000000001E-4" maxValue="0.83050000000000002"/>
     </cacheField>
     <cacheField name="Precio Ejecutado" numFmtId="6">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1" maxValue="1656.828"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1" maxValue="1661.83049999999"/>
     </cacheField>
     <cacheField name="Precio total" numFmtId="6">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-1468496.8415325161" maxValue="10000000"/>
     </cacheField>
     <cacheField name="Days (Fecha)" numFmtId="0" databaseField="0">
       <fieldGroup base="0">
-        <rangePr groupBy="days" startDate="2026-03-11T00:00:00" endDate="2026-05-02T00:00:00"/>
+        <rangePr groupBy="days" startDate="2026-03-11T00:00:00" endDate="2026-05-09T00:00:00"/>
         <groupItems count="368">
           <s v="&lt;11/03/2026"/>
           <s v="01-ene"/>
@@ -793,13 +793,13 @@
           <s v="29-dic"/>
           <s v="30-dic"/>
           <s v="31-dic"/>
-          <s v="&gt;02/05/2026"/>
+          <s v="&gt;09/05/2026"/>
         </groupItems>
       </fieldGroup>
     </cacheField>
     <cacheField name="Months (Fecha)" numFmtId="0" databaseField="0">
       <fieldGroup base="0">
-        <rangePr groupBy="months" startDate="2026-03-11T00:00:00" endDate="2026-05-02T00:00:00"/>
+        <rangePr groupBy="months" startDate="2026-03-11T00:00:00" endDate="2026-05-09T00:00:00"/>
         <groupItems count="14">
           <s v="&lt;11/03/2026"/>
           <s v="ene"/>
@@ -814,7 +814,7 @@
           <s v="oct"/>
           <s v="nov"/>
           <s v="dic"/>
-          <s v="&gt;02/05/2026"/>
+          <s v="&gt;09/05/2026"/>
         </groupItems>
       </fieldGroup>
     </cacheField>
@@ -828,7 +828,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="145">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="161">
   <r>
     <x v="0"/>
     <x v="0"/>
@@ -2279,12 +2279,172 @@
     <n v="57.101436067581098"/>
     <n v="215786.32689938898"/>
   </r>
+  <r>
+    <x v="9"/>
+    <x v="4"/>
+    <s v="COMPRA"/>
+    <n v="2022"/>
+    <n v="146.850006103515"/>
+    <n v="7.3425003051757795E-2"/>
+    <n v="146.92343110656699"/>
+    <n v="-297079.17769747844"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="17"/>
+    <s v="COMPRA"/>
+    <n v="32"/>
+    <n v="1661"/>
+    <n v="0.83050000000000002"/>
+    <n v="1661.83049999999"/>
+    <n v="-53178.575999999681"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="9"/>
+    <s v="COMPRA"/>
+    <n v="3709"/>
+    <n v="61.900001525878899"/>
+    <n v="3.0950000762939401E-2"/>
+    <n v="61.930951526641799"/>
+    <n v="-229701.89921231443"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="5"/>
+    <s v="COMPRA"/>
+    <n v="2471"/>
+    <n v="41.009998321533203"/>
+    <n v="2.0504999160766601E-2"/>
+    <n v="41.030503320693903"/>
+    <n v="-101386.37370543463"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="20"/>
+    <s v="COMPRA"/>
+    <n v="8778"/>
+    <n v="61.659999847412102"/>
+    <n v="3.0829999923706001E-2"/>
+    <n v="61.690829847335799"/>
+    <n v="-541522.10439991369"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="25"/>
+    <s v="COMPRA"/>
+    <n v="22827"/>
+    <n v="10.465999603271401"/>
+    <n v="5.2329998016357399E-3"/>
+    <n v="10.4712326030731"/>
+    <n v="-239026.82663034965"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="11"/>
+    <s v="COMPRA"/>
+    <n v="151"/>
+    <n v="942.79998779296795"/>
+    <n v="0.47139999389648402"/>
+    <n v="943.27138778686503"/>
+    <n v="-142433.97955581662"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="18"/>
+    <s v="COMPRA"/>
+    <n v="8816"/>
+    <n v="22.770000457763601"/>
+    <n v="1.13850002288818E-2"/>
+    <n v="22.781385457992499"/>
+    <n v="-200840.69419766188"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="13"/>
+    <s v="COMPRA"/>
+    <n v="43"/>
+    <n v="1218.40002441406"/>
+    <n v="0.60920001220703102"/>
+    <n v="1219.0092244262601"/>
+    <n v="-52417.396650329181"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="6"/>
+    <s v="COMPRA"/>
+    <n v="1148"/>
+    <n v="146.19999694824199"/>
+    <n v="7.3099998474121006E-2"/>
+    <n v="146.27309694671601"/>
+    <n v="-167921.51529482997"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="27"/>
+    <s v="VENTA"/>
+    <n v="-4104"/>
+    <n v="91.550003051757798"/>
+    <n v="4.5775001525878899E-2"/>
+    <n v="91.504228050231902"/>
+    <n v="375533.35191815172"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="2"/>
+    <s v="VENTA"/>
+    <n v="-666"/>
+    <n v="178.13999938964801"/>
+    <n v="8.9069999694824195E-2"/>
+    <n v="178.05092938995301"/>
+    <n v="118581.9189737087"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="3"/>
+    <s v="VENTA"/>
+    <n v="-26272"/>
+    <n v="18.924999237060501"/>
+    <n v="9.4624996185302696E-3"/>
+    <n v="18.915536737442"/>
+    <n v="496948.98116607621"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="12"/>
+    <s v="VENTA"/>
+    <n v="-12907"/>
+    <n v="27.165000915527301"/>
+    <n v="1.35825004577636E-2"/>
+    <n v="27.1514184150695"/>
+    <n v="350443.35748330201"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="1"/>
+    <s v="VENTA"/>
+    <n v="-148"/>
+    <n v="1319.40002441406"/>
+    <n v="0.65970001220703101"/>
+    <n v="1318.7403244018501"/>
+    <n v="195173.56801147381"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="10"/>
+    <s v="VENTA"/>
+    <n v="-10564"/>
+    <n v="36.9799995422363"/>
+    <n v="1.84899997711181E-2"/>
+    <n v="36.961509542465201"/>
+    <n v="390461.38680660236"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA75CCB5-861C-4E63-A423-1C9A4AC3CFAA}" name="PivotTable2" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="J3:K13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA75CCB5-861C-4E63-A423-1C9A4AC3CFAA}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="J3:K14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" numFmtId="14" showAll="0">
       <items count="31">
@@ -2297,13 +2457,13 @@
         <item x="6"/>
         <item x="7"/>
         <item x="8"/>
-        <item m="1" x="9"/>
         <item m="1" x="10"/>
         <item m="1" x="11"/>
         <item m="1" x="12"/>
         <item m="1" x="13"/>
         <item m="1" x="14"/>
         <item m="1" x="15"/>
+        <item x="9"/>
         <item m="1" x="16"/>
         <item m="1" x="17"/>
         <item m="1" x="18"/>
@@ -2724,7 +2884,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="10">
+  <rowItems count="11">
     <i>
       <x/>
     </i>
@@ -2752,6 +2912,9 @@
     <i>
       <x v="8"/>
     </i>
+    <i>
+      <x v="15"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
@@ -2775,8 +2938,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98EFF2E4-313D-4FF3-8D4A-C66D4400DAC9}" name="PivotTable1" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="J17:AM28" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98EFF2E4-313D-4FF3-8D4A-C66D4400DAC9}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="J17:AM29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" numFmtId="14" showAll="0">
       <items count="31">
@@ -2789,13 +2952,13 @@
         <item x="6"/>
         <item x="7"/>
         <item x="8"/>
-        <item m="1" x="9"/>
         <item m="1" x="10"/>
         <item m="1" x="11"/>
         <item m="1" x="12"/>
         <item m="1" x="13"/>
         <item m="1" x="14"/>
         <item m="1" x="15"/>
+        <item x="9"/>
         <item m="1" x="16"/>
         <item m="1" x="17"/>
         <item m="1" x="18"/>
@@ -2813,7 +2976,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisCol" showAll="0">
+    <pivotField axis="axisCol" showAll="0" sortType="ascending">
       <items count="29">
         <item x="4"/>
         <item x="11"/>
@@ -2822,6 +2985,7 @@
         <item x="1"/>
         <item x="10"/>
         <item x="3"/>
+        <item x="27"/>
         <item x="0"/>
         <item x="12"/>
         <item x="7"/>
@@ -2842,7 +3006,6 @@
         <item x="21"/>
         <item x="22"/>
         <item x="9"/>
-        <item x="27"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -3248,7 +3411,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="10">
+  <rowItems count="11">
     <i>
       <x/>
     </i>
@@ -3275,6 +3438,9 @@
     </i>
     <i>
       <x v="8"/>
+    </i>
+    <i>
+      <x v="15"/>
     </i>
     <i t="grand">
       <x/>
@@ -3388,8 +3554,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:H146" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:H146" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}" name="Operaciones_table" displayName="Operaciones_table" ref="A1:H162" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:H162" xr:uid="{AF3EA3D0-E1A3-419B-913B-26162BBCD494}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{44FA3C79-852A-4F12-92D9-096D28BC8418}" name="Fecha" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{F91244B1-0D90-49D6-8C5E-74710714DBAE}" name="ID"/>
@@ -3629,7 +3795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM146"/>
+  <dimension ref="A1:AM162"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.875" bestFit="1" customWidth="1"/>
@@ -3642,27 +3808,27 @@
     <col min="14" max="15" width="9.375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.25" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="7.625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.25" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7.875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="8" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="8.375" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="12.5" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="8.375" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="11.875" bestFit="1" customWidth="1"/>
@@ -4114,11 +4280,11 @@
         <v>-666625.7598</v>
       </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="7" t="s">
-        <v>40</v>
+      <c r="J13" s="7">
+        <v>46150</v>
       </c>
       <c r="K13" s="2">
-        <v>-3032.7167311359517</v>
+        <v>-98365.97898481373</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -4148,6 +4314,12 @@
         <v>-666656.70629999996</v>
       </c>
       <c r="I14" s="2"/>
+      <c r="J14" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" s="2">
+        <v>-101398.69571594968</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
@@ -4294,67 +4466,67 @@
         <v>7</v>
       </c>
       <c r="R18" t="s">
+        <v>45</v>
+      </c>
+      <c r="S18" t="s">
         <v>29</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T18" t="s">
         <v>16</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U18" t="s">
         <v>11</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V18" t="s">
         <v>25</v>
       </c>
-      <c r="V18" t="s">
+      <c r="W18" t="s">
         <v>6</v>
       </c>
-      <c r="W18" t="s">
+      <c r="X18" t="s">
         <v>32</v>
       </c>
-      <c r="X18" t="s">
+      <c r="Y18" t="s">
         <v>36</v>
       </c>
-      <c r="Y18" t="s">
+      <c r="Z18" t="s">
         <v>38</v>
       </c>
-      <c r="Z18" t="s">
+      <c r="AA18" t="s">
         <v>20</v>
       </c>
-      <c r="AA18" t="s">
+      <c r="AB18" t="s">
         <v>9</v>
       </c>
-      <c r="AB18" t="s">
+      <c r="AC18" t="s">
         <v>12</v>
       </c>
-      <c r="AC18" t="s">
+      <c r="AD18" t="s">
         <v>17</v>
       </c>
-      <c r="AD18" t="s">
+      <c r="AE18" t="s">
         <v>27</v>
       </c>
-      <c r="AE18" t="s">
+      <c r="AF18" t="s">
         <v>35</v>
       </c>
-      <c r="AF18" t="s">
+      <c r="AG18" t="s">
         <v>37</v>
       </c>
-      <c r="AG18" t="s">
+      <c r="AH18" t="s">
         <v>10</v>
       </c>
-      <c r="AH18" t="s">
+      <c r="AI18" t="s">
         <v>28</v>
       </c>
-      <c r="AI18" t="s">
+      <c r="AJ18" t="s">
         <v>33</v>
       </c>
-      <c r="AJ18" t="s">
+      <c r="AK18" t="s">
         <v>34</v>
       </c>
-      <c r="AK18" t="s">
+      <c r="AL18" t="s">
         <v>13</v>
-      </c>
-      <c r="AL18" t="s">
-        <v>45</v>
       </c>
       <c r="AM18" t="s">
         <v>40</v>
@@ -4396,10 +4568,10 @@
       <c r="O19" s="10"/>
       <c r="P19" s="10"/>
       <c r="Q19" s="10"/>
-      <c r="R19" s="10">
+      <c r="R19" s="10"/>
+      <c r="S19" s="10">
         <v>-10000000</v>
       </c>
-      <c r="S19" s="10"/>
       <c r="T19" s="10"/>
       <c r="U19" s="10"/>
       <c r="V19" s="10"/>
@@ -4474,44 +4646,44 @@
         <v>36623</v>
       </c>
       <c r="R20" s="10"/>
-      <c r="S20" s="10">
+      <c r="S20" s="10"/>
+      <c r="T20" s="10">
         <v>25909</v>
       </c>
-      <c r="T20" s="10">
+      <c r="U20" s="10">
         <v>3159</v>
       </c>
-      <c r="U20" s="10"/>
-      <c r="V20" s="10">
+      <c r="V20" s="10"/>
+      <c r="W20" s="10">
         <v>4362</v>
       </c>
-      <c r="W20" s="10"/>
       <c r="X20" s="10"/>
       <c r="Y20" s="10"/>
-      <c r="Z20" s="10">
+      <c r="Z20" s="10"/>
+      <c r="AA20" s="10">
         <v>366.96075312617717</v>
       </c>
-      <c r="AA20" s="10">
+      <c r="AB20" s="10">
         <v>14659</v>
       </c>
-      <c r="AB20" s="10">
+      <c r="AC20" s="10">
         <v>2276</v>
       </c>
-      <c r="AC20" s="10">
+      <c r="AD20" s="10">
         <v>429</v>
       </c>
-      <c r="AD20" s="10"/>
       <c r="AE20" s="10"/>
       <c r="AF20" s="10"/>
-      <c r="AG20" s="10">
+      <c r="AG20" s="10"/>
+      <c r="AH20" s="10">
         <v>3987</v>
       </c>
-      <c r="AH20" s="10"/>
       <c r="AI20" s="10"/>
       <c r="AJ20" s="10"/>
-      <c r="AK20" s="10">
+      <c r="AK20" s="10"/>
+      <c r="AL20" s="10">
         <v>9919</v>
       </c>
-      <c r="AL20" s="10"/>
       <c r="AM20" s="10">
         <v>129667.96075312617</v>
       </c>
@@ -4567,48 +4739,48 @@
         <v>-36623</v>
       </c>
       <c r="R21" s="10"/>
-      <c r="S21" s="10">
+      <c r="S21" s="10"/>
+      <c r="T21" s="10">
         <v>-472</v>
       </c>
-      <c r="T21" s="10">
+      <c r="U21" s="10">
         <v>74</v>
       </c>
-      <c r="U21" s="10">
+      <c r="V21" s="10">
         <v>26650</v>
       </c>
-      <c r="V21" s="10">
+      <c r="W21" s="10">
         <v>112</v>
       </c>
-      <c r="W21" s="10"/>
       <c r="X21" s="10"/>
       <c r="Y21" s="10"/>
       <c r="Z21" s="10"/>
-      <c r="AA21" s="10">
+      <c r="AA21" s="10"/>
+      <c r="AB21" s="10">
         <v>1077</v>
       </c>
-      <c r="AB21" s="10">
+      <c r="AC21" s="10">
         <v>24</v>
       </c>
-      <c r="AC21" s="10">
+      <c r="AD21" s="10">
         <v>-429</v>
       </c>
-      <c r="AD21" s="10">
+      <c r="AE21" s="10">
         <v>380</v>
       </c>
-      <c r="AE21" s="10"/>
       <c r="AF21" s="10"/>
-      <c r="AG21" s="10">
+      <c r="AG21" s="10"/>
+      <c r="AH21" s="10">
         <v>107</v>
       </c>
-      <c r="AH21" s="10">
+      <c r="AI21" s="10">
         <v>9246</v>
       </c>
-      <c r="AI21" s="10"/>
       <c r="AJ21" s="10"/>
-      <c r="AK21" s="10">
+      <c r="AK21" s="10"/>
+      <c r="AL21" s="10">
         <v>-294</v>
       </c>
-      <c r="AL21" s="10"/>
       <c r="AM21" s="10">
         <v>-4636</v>
       </c>
@@ -4660,60 +4832,60 @@
       </c>
       <c r="Q22" s="10"/>
       <c r="R22" s="10"/>
-      <c r="S22" s="10">
+      <c r="S22" s="10"/>
+      <c r="T22" s="10">
         <v>-13938</v>
       </c>
-      <c r="T22" s="10">
+      <c r="U22" s="10">
         <v>-3233</v>
       </c>
-      <c r="U22" s="10">
+      <c r="V22" s="10">
         <v>34714</v>
       </c>
-      <c r="V22" s="10">
+      <c r="W22" s="10">
         <v>-321</v>
       </c>
-      <c r="W22" s="10">
+      <c r="X22" s="10">
         <v>5846</v>
       </c>
-      <c r="X22" s="10">
+      <c r="Y22" s="10">
         <v>34709</v>
       </c>
-      <c r="Y22" s="10"/>
       <c r="Z22" s="10"/>
-      <c r="AA22" s="10">
+      <c r="AA22" s="10"/>
+      <c r="AB22" s="10">
         <v>-15736</v>
       </c>
-      <c r="AB22" s="10">
+      <c r="AC22" s="10">
         <v>-2300</v>
       </c>
-      <c r="AC22" s="10">
+      <c r="AD22" s="10">
         <v>221</v>
       </c>
-      <c r="AD22" s="10">
+      <c r="AE22" s="10">
         <v>-380</v>
       </c>
-      <c r="AE22" s="10">
+      <c r="AF22" s="10">
         <v>1724</v>
       </c>
-      <c r="AF22" s="10">
+      <c r="AG22" s="10">
         <v>56041</v>
       </c>
-      <c r="AG22" s="10">
+      <c r="AH22" s="10">
         <v>-4094</v>
       </c>
-      <c r="AH22" s="10">
+      <c r="AI22" s="10">
         <v>-1553</v>
       </c>
-      <c r="AI22" s="10">
+      <c r="AJ22" s="10">
         <v>18700</v>
       </c>
-      <c r="AJ22" s="10">
+      <c r="AK22" s="10">
         <v>12173</v>
       </c>
-      <c r="AK22" s="10">
+      <c r="AL22" s="10">
         <v>-9625</v>
       </c>
-      <c r="AL22" s="10"/>
       <c r="AM22" s="10">
         <v>107265</v>
       </c>
@@ -4763,49 +4935,49 @@
         <v>37957</v>
       </c>
       <c r="R23" s="10"/>
-      <c r="S23" s="10">
+      <c r="S23" s="10"/>
+      <c r="T23" s="10">
         <v>1216</v>
       </c>
-      <c r="T23" s="10"/>
-      <c r="U23" s="10">
+      <c r="U23" s="10"/>
+      <c r="V23" s="10">
         <v>-12852</v>
       </c>
-      <c r="V23" s="10">
+      <c r="W23" s="10">
         <v>-2461</v>
       </c>
-      <c r="W23" s="10">
+      <c r="X23" s="10">
         <v>6143</v>
       </c>
-      <c r="X23" s="10">
+      <c r="Y23" s="10">
         <v>-5905</v>
       </c>
-      <c r="Y23" s="10"/>
       <c r="Z23" s="10"/>
       <c r="AA23" s="10"/>
-      <c r="AB23" s="10">
+      <c r="AB23" s="10"/>
+      <c r="AC23" s="10">
         <v>782</v>
       </c>
-      <c r="AC23" s="10">
+      <c r="AD23" s="10">
         <v>-221</v>
       </c>
-      <c r="AD23" s="10"/>
-      <c r="AE23" s="10">
+      <c r="AE23" s="10"/>
+      <c r="AF23" s="10">
         <v>246</v>
       </c>
-      <c r="AF23" s="10">
+      <c r="AG23" s="10">
         <v>-4227</v>
       </c>
-      <c r="AG23" s="10"/>
-      <c r="AH23" s="10">
+      <c r="AH23" s="10"/>
+      <c r="AI23" s="10">
         <v>-3861</v>
       </c>
-      <c r="AI23" s="10">
+      <c r="AJ23" s="10">
         <v>2177</v>
       </c>
-      <c r="AJ23" s="10">
+      <c r="AK23" s="10">
         <v>-12173</v>
       </c>
-      <c r="AK23" s="10"/>
       <c r="AL23" s="10"/>
       <c r="AM23" s="10">
         <v>15410</v>
@@ -4858,44 +5030,44 @@
         <v>-36557</v>
       </c>
       <c r="R24" s="10"/>
-      <c r="S24" s="10">
+      <c r="S24" s="10"/>
+      <c r="T24" s="10">
         <v>663</v>
       </c>
-      <c r="T24" s="10"/>
-      <c r="U24" s="10">
+      <c r="U24" s="10"/>
+      <c r="V24" s="10">
         <v>-3328</v>
       </c>
-      <c r="V24" s="10">
+      <c r="W24" s="10">
         <v>6951</v>
       </c>
-      <c r="W24" s="10">
+      <c r="X24" s="10">
         <v>-2481</v>
       </c>
-      <c r="X24" s="10"/>
       <c r="Y24" s="10"/>
       <c r="Z24" s="10"/>
-      <c r="AA24" s="10">
+      <c r="AA24" s="10"/>
+      <c r="AB24" s="10">
         <v>2584</v>
       </c>
-      <c r="AB24" s="10">
+      <c r="AC24" s="10">
         <v>-115</v>
       </c>
-      <c r="AC24" s="10"/>
       <c r="AD24" s="10"/>
-      <c r="AE24" s="10">
+      <c r="AE24" s="10"/>
+      <c r="AF24" s="10">
         <v>-400</v>
       </c>
-      <c r="AF24" s="10">
+      <c r="AG24" s="10">
         <v>19597</v>
       </c>
-      <c r="AG24" s="10"/>
-      <c r="AH24" s="10">
+      <c r="AH24" s="10"/>
+      <c r="AI24" s="10">
         <v>-3049</v>
       </c>
-      <c r="AI24" s="10">
+      <c r="AJ24" s="10">
         <v>3599</v>
       </c>
-      <c r="AJ24" s="10"/>
       <c r="AK24" s="10"/>
       <c r="AL24" s="10"/>
       <c r="AM24" s="10">
@@ -4949,52 +5121,52 @@
         <v>832</v>
       </c>
       <c r="R25" s="10"/>
-      <c r="S25" s="10">
+      <c r="S25" s="10"/>
+      <c r="T25" s="10">
         <v>6891</v>
       </c>
-      <c r="T25" s="10"/>
-      <c r="U25" s="10">
+      <c r="U25" s="10"/>
+      <c r="V25" s="10">
         <v>-938</v>
       </c>
-      <c r="V25" s="10">
+      <c r="W25" s="10">
         <v>-4228</v>
       </c>
-      <c r="W25" s="10">
+      <c r="X25" s="10">
         <v>-6028</v>
       </c>
-      <c r="X25" s="10"/>
-      <c r="Y25" s="10">
+      <c r="Y25" s="10"/>
+      <c r="Z25" s="10">
         <v>4327</v>
       </c>
-      <c r="Z25" s="10"/>
-      <c r="AA25" s="10">
+      <c r="AA25" s="10"/>
+      <c r="AB25" s="10">
         <v>-803</v>
       </c>
-      <c r="AB25" s="10">
+      <c r="AC25" s="10">
         <v>-1010</v>
       </c>
-      <c r="AC25" s="10"/>
       <c r="AD25" s="10"/>
-      <c r="AE25" s="10">
+      <c r="AE25" s="10"/>
+      <c r="AF25" s="10">
         <v>-1147</v>
       </c>
-      <c r="AF25" s="10">
+      <c r="AG25" s="10">
         <v>-50484</v>
       </c>
-      <c r="AG25" s="10">
+      <c r="AH25" s="10">
         <v>1388</v>
       </c>
-      <c r="AH25" s="10">
+      <c r="AI25" s="10">
         <v>-1765</v>
       </c>
-      <c r="AI25" s="10">
+      <c r="AJ25" s="10">
         <v>2329</v>
       </c>
-      <c r="AJ25" s="10"/>
-      <c r="AK25" s="10">
+      <c r="AK25" s="10"/>
+      <c r="AL25" s="10">
         <v>3946</v>
       </c>
-      <c r="AL25" s="10"/>
       <c r="AM25" s="10">
         <v>-28364</v>
       </c>
@@ -5046,50 +5218,50 @@
         <v>9644</v>
       </c>
       <c r="R26" s="10"/>
-      <c r="S26" s="10">
+      <c r="S26" s="10"/>
+      <c r="T26" s="10">
         <v>-7468</v>
       </c>
-      <c r="T26" s="10"/>
-      <c r="U26" s="10">
+      <c r="U26" s="10"/>
+      <c r="V26" s="10">
         <v>10225</v>
       </c>
-      <c r="V26" s="10">
+      <c r="W26" s="10">
         <v>3623</v>
       </c>
-      <c r="W26" s="10">
+      <c r="X26" s="10">
         <v>11124</v>
       </c>
-      <c r="X26" s="10"/>
-      <c r="Y26" s="10">
+      <c r="Y26" s="10"/>
+      <c r="Z26" s="10">
         <v>23473</v>
       </c>
-      <c r="Z26" s="10"/>
-      <c r="AA26" s="10">
+      <c r="AA26" s="10"/>
+      <c r="AB26" s="10">
         <v>2251</v>
       </c>
-      <c r="AB26" s="10"/>
-      <c r="AC26" s="10">
+      <c r="AC26" s="10"/>
+      <c r="AD26" s="10">
         <v>225</v>
       </c>
-      <c r="AD26" s="10"/>
-      <c r="AE26" s="10">
+      <c r="AE26" s="10"/>
+      <c r="AF26" s="10">
         <v>-1247</v>
       </c>
-      <c r="AF26" s="10"/>
-      <c r="AG26" s="10">
+      <c r="AG26" s="10"/>
+      <c r="AH26" s="10">
         <v>208</v>
       </c>
-      <c r="AH26" s="10">
+      <c r="AI26" s="10">
         <v>-1055</v>
       </c>
-      <c r="AI26" s="10">
+      <c r="AJ26" s="10">
         <v>-22074</v>
       </c>
-      <c r="AJ26" s="10"/>
-      <c r="AK26" s="10">
+      <c r="AK26" s="10"/>
+      <c r="AL26" s="10">
         <v>1059</v>
       </c>
-      <c r="AL26" s="10"/>
       <c r="AM26" s="10">
         <v>1985</v>
       </c>
@@ -5140,60 +5312,60 @@
       <c r="Q27" s="10">
         <v>26551</v>
       </c>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10">
+      <c r="R27" s="10">
+        <v>4104</v>
+      </c>
+      <c r="S27" s="10"/>
+      <c r="T27" s="10">
         <v>11411</v>
       </c>
-      <c r="T27" s="10"/>
-      <c r="U27" s="10">
+      <c r="U27" s="10"/>
+      <c r="V27" s="10">
         <v>9077</v>
       </c>
-      <c r="V27" s="10">
+      <c r="W27" s="10">
         <v>380</v>
       </c>
-      <c r="W27" s="10">
+      <c r="X27" s="10">
         <v>-3779</v>
       </c>
-      <c r="X27" s="10">
+      <c r="Y27" s="10">
         <v>-28804</v>
       </c>
-      <c r="Y27" s="10">
+      <c r="Z27" s="10">
         <v>-27800</v>
       </c>
-      <c r="Z27" s="10"/>
-      <c r="AA27" s="10">
+      <c r="AA27" s="10"/>
+      <c r="AB27" s="10">
         <v>1204</v>
       </c>
-      <c r="AB27" s="10">
+      <c r="AC27" s="10">
         <v>343</v>
       </c>
-      <c r="AC27" s="10">
+      <c r="AD27" s="10">
         <v>-7</v>
       </c>
-      <c r="AD27" s="10">
+      <c r="AE27" s="10">
         <v>130</v>
       </c>
-      <c r="AE27" s="10">
+      <c r="AF27" s="10">
         <v>824</v>
       </c>
-      <c r="AF27" s="10">
+      <c r="AG27" s="10">
         <v>14533</v>
       </c>
-      <c r="AG27" s="10">
+      <c r="AH27" s="10">
         <v>-96</v>
       </c>
-      <c r="AH27" s="10">
+      <c r="AI27" s="10">
         <v>2037</v>
       </c>
-      <c r="AI27" s="10">
+      <c r="AJ27" s="10">
         <v>-4731</v>
       </c>
-      <c r="AJ27" s="10"/>
-      <c r="AK27" s="10">
+      <c r="AK27" s="10"/>
+      <c r="AL27" s="10">
         <v>-1215</v>
-      </c>
-      <c r="AL27" s="10">
-        <v>4104</v>
       </c>
       <c r="AM27" s="10">
         <v>17482</v>
@@ -5225,95 +5397,71 @@
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>-629782.43077839643</v>
       </c>
-      <c r="J28" s="7" t="s">
-        <v>40</v>
+      <c r="J28" s="7">
+        <v>46150</v>
       </c>
       <c r="K28" s="10">
-        <v>0</v>
+        <v>2022</v>
       </c>
       <c r="L28" s="10">
-        <v>245</v>
-      </c>
-      <c r="M28" s="10">
-        <v>0</v>
-      </c>
-      <c r="N28" s="10">
-        <v>0</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
       <c r="O28" s="10">
-        <v>1247</v>
+        <v>-148</v>
       </c>
       <c r="P28" s="10">
-        <v>35388</v>
+        <v>-10564</v>
       </c>
       <c r="Q28" s="10">
-        <v>38427</v>
+        <v>-26272</v>
       </c>
       <c r="R28" s="10">
-        <v>-10000000</v>
-      </c>
-      <c r="S28" s="10">
-        <v>24212</v>
-      </c>
+        <v>-4104</v>
+      </c>
+      <c r="S28" s="10"/>
       <c r="T28" s="10">
-        <v>0</v>
-      </c>
-      <c r="U28" s="10">
-        <v>63548</v>
-      </c>
+        <v>-12907</v>
+      </c>
+      <c r="U28" s="10"/>
       <c r="V28" s="10">
-        <v>8418</v>
+        <v>8816</v>
       </c>
       <c r="W28" s="10">
-        <v>10825</v>
+        <v>-666</v>
       </c>
       <c r="X28" s="10">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z28" s="10">
-        <v>366.96075312617717</v>
-      </c>
-      <c r="AA28" s="10">
-        <v>5236</v>
-      </c>
+        <v>8778</v>
+      </c>
+      <c r="Y28" s="10"/>
+      <c r="Z28" s="10"/>
+      <c r="AA28" s="10"/>
       <c r="AB28" s="10">
-        <v>0</v>
-      </c>
-      <c r="AC28" s="10">
-        <v>218</v>
-      </c>
+        <v>2471</v>
+      </c>
+      <c r="AC28" s="10"/>
       <c r="AD28" s="10">
-        <v>130</v>
+        <v>43</v>
       </c>
       <c r="AE28" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF28" s="10">
-        <v>35460</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="AF28" s="10"/>
       <c r="AG28" s="10">
-        <v>1500</v>
+        <v>22827</v>
       </c>
       <c r="AH28" s="10">
-        <v>0</v>
-      </c>
-      <c r="AI28" s="10">
-        <v>0</v>
-      </c>
-      <c r="AJ28" s="10">
-        <v>0</v>
-      </c>
-      <c r="AK28" s="10">
-        <v>3790</v>
-      </c>
+        <v>1148</v>
+      </c>
+      <c r="AI28" s="10"/>
+      <c r="AJ28" s="10"/>
+      <c r="AK28" s="10"/>
       <c r="AL28" s="10">
-        <v>4104</v>
+        <v>3709</v>
       </c>
       <c r="AM28" s="10">
-        <v>-9766885.0392468739</v>
+        <v>-4664</v>
       </c>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
@@ -5342,6 +5490,96 @@
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>19229.741037414537</v>
       </c>
+      <c r="J29" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K29" s="10">
+        <v>2022</v>
+      </c>
+      <c r="L29" s="10">
+        <v>396</v>
+      </c>
+      <c r="M29" s="10">
+        <v>0</v>
+      </c>
+      <c r="N29" s="10">
+        <v>0</v>
+      </c>
+      <c r="O29" s="10">
+        <v>1099</v>
+      </c>
+      <c r="P29" s="10">
+        <v>24824</v>
+      </c>
+      <c r="Q29" s="10">
+        <v>12155</v>
+      </c>
+      <c r="R29" s="10">
+        <v>0</v>
+      </c>
+      <c r="S29" s="10">
+        <v>-10000000</v>
+      </c>
+      <c r="T29" s="10">
+        <v>11305</v>
+      </c>
+      <c r="U29" s="10">
+        <v>0</v>
+      </c>
+      <c r="V29" s="10">
+        <v>72364</v>
+      </c>
+      <c r="W29" s="10">
+        <v>7752</v>
+      </c>
+      <c r="X29" s="10">
+        <v>19603</v>
+      </c>
+      <c r="Y29" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="10">
+        <v>366.96075312617717</v>
+      </c>
+      <c r="AB29" s="10">
+        <v>7707</v>
+      </c>
+      <c r="AC29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="10">
+        <v>261</v>
+      </c>
+      <c r="AE29" s="10">
+        <v>162</v>
+      </c>
+      <c r="AF29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="10">
+        <v>58287</v>
+      </c>
+      <c r="AH29" s="10">
+        <v>2648</v>
+      </c>
+      <c r="AI29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AL29" s="10">
+        <v>7499</v>
+      </c>
+      <c r="AM29" s="10">
+        <v>-9771549.0392468739</v>
+      </c>
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
@@ -8500,6 +8738,438 @@
       <c r="H146" s="2">
         <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
         <v>215786.32689938898</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B147" t="s">
+        <v>8</v>
+      </c>
+      <c r="C147" t="s">
+        <v>23</v>
+      </c>
+      <c r="D147">
+        <v>2022</v>
+      </c>
+      <c r="E147" s="2">
+        <v>146.850006103515</v>
+      </c>
+      <c r="F147" s="10">
+        <v>7.3425003051757795E-2</v>
+      </c>
+      <c r="G147" s="2">
+        <v>146.92343110656699</v>
+      </c>
+      <c r="H147" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-297079.17769747844</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B148" t="s">
+        <v>27</v>
+      </c>
+      <c r="C148" t="s">
+        <v>23</v>
+      </c>
+      <c r="D148">
+        <v>32</v>
+      </c>
+      <c r="E148" s="2">
+        <v>1661</v>
+      </c>
+      <c r="F148" s="10">
+        <v>0.83050000000000002</v>
+      </c>
+      <c r="G148" s="2">
+        <v>1661.83049999999</v>
+      </c>
+      <c r="H148" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-53178.575999999681</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B149" t="s">
+        <v>13</v>
+      </c>
+      <c r="C149" t="s">
+        <v>23</v>
+      </c>
+      <c r="D149">
+        <v>3709</v>
+      </c>
+      <c r="E149" s="2">
+        <v>61.900001525878899</v>
+      </c>
+      <c r="F149" s="10">
+        <v>3.0950000762939401E-2</v>
+      </c>
+      <c r="G149" s="2">
+        <v>61.930951526641799</v>
+      </c>
+      <c r="H149" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-229701.89921231443</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B150" t="s">
+        <v>9</v>
+      </c>
+      <c r="C150" t="s">
+        <v>23</v>
+      </c>
+      <c r="D150">
+        <v>2471</v>
+      </c>
+      <c r="E150" s="2">
+        <v>41.009998321533203</v>
+      </c>
+      <c r="F150" s="10">
+        <v>2.0504999160766601E-2</v>
+      </c>
+      <c r="G150" s="2">
+        <v>41.030503320693903</v>
+      </c>
+      <c r="H150" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-101386.37370543463</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>32</v>
+      </c>
+      <c r="C151" t="s">
+        <v>23</v>
+      </c>
+      <c r="D151">
+        <v>8778</v>
+      </c>
+      <c r="E151" s="2">
+        <v>61.659999847412102</v>
+      </c>
+      <c r="F151" s="10">
+        <v>3.0829999923706001E-2</v>
+      </c>
+      <c r="G151" s="2">
+        <v>61.690829847335799</v>
+      </c>
+      <c r="H151" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-541522.10439991369</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B152" t="s">
+        <v>37</v>
+      </c>
+      <c r="C152" t="s">
+        <v>23</v>
+      </c>
+      <c r="D152">
+        <v>22827</v>
+      </c>
+      <c r="E152" s="2">
+        <v>10.465999603271401</v>
+      </c>
+      <c r="F152" s="10">
+        <v>5.2329998016357399E-3</v>
+      </c>
+      <c r="G152" s="2">
+        <v>10.4712326030731</v>
+      </c>
+      <c r="H152" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-239026.82663034965</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B153" t="s">
+        <v>15</v>
+      </c>
+      <c r="C153" t="s">
+        <v>23</v>
+      </c>
+      <c r="D153">
+        <v>151</v>
+      </c>
+      <c r="E153" s="2">
+        <v>942.79998779296795</v>
+      </c>
+      <c r="F153" s="10">
+        <v>0.47139999389648402</v>
+      </c>
+      <c r="G153" s="2">
+        <v>943.27138778686503</v>
+      </c>
+      <c r="H153" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-142433.97955581662</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B154" t="s">
+        <v>25</v>
+      </c>
+      <c r="C154" t="s">
+        <v>23</v>
+      </c>
+      <c r="D154">
+        <v>8816</v>
+      </c>
+      <c r="E154" s="2">
+        <v>22.770000457763601</v>
+      </c>
+      <c r="F154" s="10">
+        <v>1.13850002288818E-2</v>
+      </c>
+      <c r="G154" s="2">
+        <v>22.781385457992499</v>
+      </c>
+      <c r="H154" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-200840.69419766188</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B155" t="s">
+        <v>17</v>
+      </c>
+      <c r="C155" t="s">
+        <v>23</v>
+      </c>
+      <c r="D155">
+        <v>43</v>
+      </c>
+      <c r="E155" s="2">
+        <v>1218.40002441406</v>
+      </c>
+      <c r="F155" s="10">
+        <v>0.60920001220703102</v>
+      </c>
+      <c r="G155" s="2">
+        <v>1219.0092244262601</v>
+      </c>
+      <c r="H155" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-52417.396650329181</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B156" t="s">
+        <v>10</v>
+      </c>
+      <c r="C156" t="s">
+        <v>23</v>
+      </c>
+      <c r="D156">
+        <v>1148</v>
+      </c>
+      <c r="E156" s="2">
+        <v>146.19999694824199</v>
+      </c>
+      <c r="F156" s="10">
+        <v>7.3099998474121006E-2</v>
+      </c>
+      <c r="G156" s="2">
+        <v>146.27309694671601</v>
+      </c>
+      <c r="H156" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>-167921.51529482997</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B157" t="s">
+        <v>45</v>
+      </c>
+      <c r="C157" t="s">
+        <v>26</v>
+      </c>
+      <c r="D157">
+        <v>-4104</v>
+      </c>
+      <c r="E157" s="2">
+        <v>91.550003051757798</v>
+      </c>
+      <c r="F157" s="10">
+        <v>4.5775001525878899E-2</v>
+      </c>
+      <c r="G157" s="2">
+        <v>91.504228050231902</v>
+      </c>
+      <c r="H157" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>375533.35191815172</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B158" t="s">
+        <v>6</v>
+      </c>
+      <c r="C158" t="s">
+        <v>26</v>
+      </c>
+      <c r="D158">
+        <v>-666</v>
+      </c>
+      <c r="E158" s="2">
+        <v>178.13999938964801</v>
+      </c>
+      <c r="F158" s="10">
+        <v>8.9069999694824195E-2</v>
+      </c>
+      <c r="G158" s="2">
+        <v>178.05092938995301</v>
+      </c>
+      <c r="H158" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>118581.9189737087</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B159" t="s">
+        <v>7</v>
+      </c>
+      <c r="C159" t="s">
+        <v>26</v>
+      </c>
+      <c r="D159">
+        <v>-26272</v>
+      </c>
+      <c r="E159" s="2">
+        <v>18.924999237060501</v>
+      </c>
+      <c r="F159" s="10">
+        <v>9.4624996185302696E-3</v>
+      </c>
+      <c r="G159" s="2">
+        <v>18.915536737442</v>
+      </c>
+      <c r="H159" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>496948.98116607621</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B160" t="s">
+        <v>16</v>
+      </c>
+      <c r="C160" t="s">
+        <v>26</v>
+      </c>
+      <c r="D160">
+        <v>-12907</v>
+      </c>
+      <c r="E160" s="2">
+        <v>27.165000915527301</v>
+      </c>
+      <c r="F160" s="10">
+        <v>1.35825004577636E-2</v>
+      </c>
+      <c r="G160" s="2">
+        <v>27.1514184150695</v>
+      </c>
+      <c r="H160" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>350443.35748330201</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B161" t="s">
+        <v>5</v>
+      </c>
+      <c r="C161" t="s">
+        <v>26</v>
+      </c>
+      <c r="D161">
+        <v>-148</v>
+      </c>
+      <c r="E161" s="2">
+        <v>1319.40002441406</v>
+      </c>
+      <c r="F161" s="10">
+        <v>0.65970001220703101</v>
+      </c>
+      <c r="G161" s="2">
+        <v>1318.7403244018501</v>
+      </c>
+      <c r="H161" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>195173.56801147381</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" s="4">
+        <v>46150</v>
+      </c>
+      <c r="B162" t="s">
+        <v>14</v>
+      </c>
+      <c r="C162" t="s">
+        <v>26</v>
+      </c>
+      <c r="D162">
+        <v>-10564</v>
+      </c>
+      <c r="E162" s="2">
+        <v>36.9799995422363</v>
+      </c>
+      <c r="F162" s="10">
+        <v>1.84899997711181E-2</v>
+      </c>
+      <c r="G162" s="2">
+        <v>36.961509542465201</v>
+      </c>
+      <c r="H162" s="2">
+        <f>-Operaciones_table[[#This Row],[Precio Ejecutado]]*Operaciones_table[[#This Row],[Cantidad]]</f>
+        <v>390461.38680660236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>